<commit_message>
pass 2, debt waterfall
</commit_message>
<xml_diff>
--- a/outputs/valuation_model.xlsx
+++ b/outputs/valuation_model.xlsx
@@ -517,7 +517,7 @@
         </is>
       </c>
       <c r="B8">
-        <f>'returns'!$B5</f>
+        <f>'returns'!$B8</f>
         <v/>
       </c>
     </row>
@@ -528,7 +528,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>'returns'!$B8</f>
+        <f>'returns'!$B12</f>
         <v/>
       </c>
     </row>
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>'returns'!$B13</f>
+        <f>'returns'!$B20</f>
         <v/>
       </c>
     </row>
@@ -550,7 +550,7 @@
         </is>
       </c>
       <c r="B11">
-        <f>'returns'!$B14</f>
+        <f>'returns'!$B21</f>
         <v/>
       </c>
     </row>
@@ -561,7 +561,7 @@
         </is>
       </c>
       <c r="B12">
-        <f>'returns'!$B15</f>
+        <f>'returns'!$B22</f>
         <v/>
       </c>
     </row>
@@ -592,7 +592,7 @@
         </is>
       </c>
       <c r="B17">
-        <f>COUNTIF(checks!C4:C11,"PASS")</f>
+        <f>COUNTIF(checks!C4:C13,"PASS")</f>
         <v/>
       </c>
     </row>
@@ -603,7 +603,7 @@
         </is>
       </c>
       <c r="B18">
-        <f>COUNTIF(checks!C4:C11,"FAIL")</f>
+        <f>COUNTIF(checks!C4:C13,"FAIL")</f>
         <v/>
       </c>
     </row>
@@ -696,7 +696,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -767,7 +767,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>MIN('debt_schedule'!$Q4,'debt_schedule'!$Q5,'debt_schedule'!$Q6,'debt_schedule'!$Q7,'debt_schedule'!$Q8)-'historicals_input'!$B19</f>
+        <f>MIN('debt_schedule'!$T4,'debt_schedule'!$T5,'debt_schedule'!$T6,'debt_schedule'!$T7,'debt_schedule'!$T8)-'historicals_input'!$B19</f>
         <v/>
       </c>
       <c r="C6">
@@ -782,7 +782,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>MIN('debt_schedule'!$R4,'debt_schedule'!$R5,'debt_schedule'!$R6,'debt_schedule'!$R7,'debt_schedule'!$R8)</f>
+        <f>MIN('debt_schedule'!$U4,'debt_schedule'!$U5,'debt_schedule'!$U6,'debt_schedule'!$U7,'debt_schedule'!$U8)</f>
         <v/>
       </c>
       <c r="C7">
@@ -797,7 +797,7 @@
         </is>
       </c>
       <c r="B8">
-        <f>MIN('debt_schedule'!$S4,'debt_schedule'!$S5,'debt_schedule'!$S6,'debt_schedule'!$S7,'debt_schedule'!$S8)</f>
+        <f>MIN('debt_schedule'!$V4,'debt_schedule'!$V5,'debt_schedule'!$V6,'debt_schedule'!$V7,'debt_schedule'!$V8)</f>
         <v/>
       </c>
       <c r="C8">
@@ -812,7 +812,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>'valuation'!$B14-'historicals_input'!$B36</f>
+        <f>'valuation'!$B14-'historicals_input'!$B38</f>
         <v/>
       </c>
       <c r="C9">
@@ -827,7 +827,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>'returns'!$B13</f>
+        <f>'returns'!$B20</f>
         <v/>
       </c>
       <c r="C10">
@@ -850,70 +850,100 @@
         <v/>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Python Safety Snapshot</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Python</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>Excel</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>Delta</t>
-        </is>
-      </c>
-    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Liquidity Shortfall = 0</t>
+        </is>
+      </c>
+      <c r="B12">
+        <f>MAX('debt_schedule'!$S4,'debt_schedule'!$S5,'debt_schedule'!$S6,'debt_schedule'!$S7,'debt_schedule'!$S8)</f>
+        <v/>
+      </c>
+      <c r="C12">
+        <f>IF(B12=0,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Revolver Within Limit</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>MAX('debt_schedule'!$W4,'debt_schedule'!$W5,'debt_schedule'!$W6,'debt_schedule'!$W7,'debt_schedule'!$W8)-'historicals_input'!$B28</f>
+        <v/>
+      </c>
+      <c r="C13">
+        <f>IF(B13&lt;=0,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>Python Safety Snapshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Delta</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>DCF Share Price (PGR)</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B18" t="n">
         <v>93.69209486764926</v>
       </c>
-      <c r="C16">
+      <c r="C18">
         <f>'valuation'!$E20</f>
         <v/>
       </c>
-      <c r="D16">
-        <f>C16-B16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="D18">
+        <f>C18-B18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>DCF Share Price (Multiple)</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B19" t="n">
         <v>91.12898270712128</v>
       </c>
-      <c r="C17">
+      <c r="C19">
         <f>'valuation'!$E21</f>
         <v/>
       </c>
-      <c r="D17">
-        <f>C17-B17</f>
+      <c r="D19">
+        <f>C19-B19</f>
         <v/>
       </c>
     </row>
@@ -928,7 +958,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -1233,88 +1263,108 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>Revolver Limit</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="n">
+        <v>6255000000</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>Senior Amortization %</t>
         </is>
       </c>
-      <c r="B28" s="5" t="n">
+      <c r="B29" s="5" t="n">
         <v>0.05</v>
       </c>
     </row>
-    <row r="29"/>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Cash Sweep %</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31"/>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>Valuation Assumptions</t>
         </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Tax Rate</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="n">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Risk Free Rate</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="n">
-        <v>0.042</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Beta</t>
-        </is>
-      </c>
-      <c r="B33" s="7" t="n">
-        <v>1.2</v>
+          <t>Tax Rate</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>0.25</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Market Risk Premium</t>
+          <t>Risk Free Rate</t>
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>0.06</v>
+        <v>0.042</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Cost of Debt</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="n">
-        <v>0.065</v>
+          <t>Beta</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="n">
+        <v>1.2</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Terminal Growth</t>
+          <t>Market Risk Premium</t>
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>0.025</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>Cost of Debt</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0.065</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Terminal Growth</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0.025</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>Exit Multiple</t>
         </is>
       </c>
-      <c r="B37" s="6" t="n">
+      <c r="B39" s="6" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1953,23 +2003,23 @@
         </is>
       </c>
       <c r="B11" s="4">
-        <f>B10*'historicals_input'!$B31</f>
+        <f>B10*'historicals_input'!$B33</f>
         <v/>
       </c>
       <c r="C11" s="4">
-        <f>C10*'historicals_input'!$B31</f>
+        <f>C10*'historicals_input'!$B33</f>
         <v/>
       </c>
       <c r="D11" s="4">
-        <f>D10*'historicals_input'!$B31</f>
+        <f>D10*'historicals_input'!$B33</f>
         <v/>
       </c>
       <c r="E11" s="4">
-        <f>E10*'historicals_input'!$B31</f>
+        <f>E10*'historicals_input'!$B33</f>
         <v/>
       </c>
       <c r="F11" s="4">
-        <f>F10*'historicals_input'!$B31</f>
+        <f>F10*'historicals_input'!$B33</f>
         <v/>
       </c>
     </row>
@@ -2146,7 +2196,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T8"/>
+  <dimension ref="A1:W8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2162,13 +2212,16 @@
     <col width="23" customWidth="1" min="11" max="11"/>
     <col width="26" customWidth="1" min="12" max="12"/>
     <col width="26" customWidth="1" min="13" max="13"/>
-    <col width="26" customWidth="1" min="14" max="14"/>
+    <col width="21" customWidth="1" min="14" max="14"/>
     <col width="26" customWidth="1" min="15" max="15"/>
-    <col width="26" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
-    <col width="18" customWidth="1" min="18" max="18"/>
-    <col width="18" customWidth="1" min="19" max="19"/>
-    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="23" customWidth="1" min="16" max="16"/>
+    <col width="26" customWidth="1" min="17" max="17"/>
+    <col width="26" customWidth="1" min="18" max="18"/>
+    <col width="26" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
+    <col width="18" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2247,35 +2300,50 @@
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
+          <t>Cash Post Mandatory</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>Cash Sweep Capacity</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
           <t>Senior Sweep</t>
         </is>
       </c>
-      <c r="O3" s="3" t="inlineStr">
+      <c r="Q3" s="3" t="inlineStr">
         <is>
           <t>Sub Sweep</t>
         </is>
       </c>
-      <c r="P3" s="3" t="inlineStr">
+      <c r="R3" s="3" t="inlineStr">
         <is>
           <t>Revolver Draw</t>
         </is>
       </c>
-      <c r="Q3" s="3" t="inlineStr">
+      <c r="S3" s="3" t="inlineStr">
+        <is>
+          <t>Liquidity Shortfall</t>
+        </is>
+      </c>
+      <c r="T3" s="3" t="inlineStr">
         <is>
           <t>End Cash</t>
         </is>
       </c>
-      <c r="R3" s="3" t="inlineStr">
+      <c r="U3" s="3" t="inlineStr">
         <is>
           <t>End Senior</t>
         </is>
       </c>
-      <c r="S3" s="3" t="inlineStr">
+      <c r="V3" s="3" t="inlineStr">
         <is>
           <t>End Sub</t>
         </is>
       </c>
-      <c r="T3" s="3" t="inlineStr">
+      <c r="W3" s="3" t="inlineStr">
         <is>
           <t>End Revolver</t>
         </is>
@@ -2285,79 +2353,91 @@
       <c r="A4" t="n">
         <v>2025</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="4">
         <f>'sources_uses'!$B9</f>
         <v/>
       </c>
-      <c r="C4">
+      <c r="C4" s="4">
         <f>'sources_uses'!$B14</f>
         <v/>
       </c>
-      <c r="D4">
+      <c r="D4" s="4">
         <f>'sources_uses'!$B15</f>
         <v/>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="4">
         <f>'operating_model'!$B17</f>
         <v/>
       </c>
-      <c r="G4">
+      <c r="G4" s="4">
         <f>C4*'historicals_input'!$B24</f>
         <v/>
       </c>
-      <c r="H4">
+      <c r="H4" s="4">
         <f>D4*'historicals_input'!$B25</f>
         <v/>
       </c>
-      <c r="I4">
+      <c r="I4" s="4">
         <f>D4*'historicals_input'!$B26</f>
         <v/>
       </c>
-      <c r="J4">
+      <c r="J4" s="4">
         <f>E4*'historicals_input'!$B27</f>
         <v/>
       </c>
-      <c r="K4">
+      <c r="K4" s="4">
         <f>B4+F4-G4-H4-J4</f>
         <v/>
       </c>
-      <c r="L4">
-        <f>MIN(C4*'historicals_input'!$B28,C4)</f>
-        <v/>
-      </c>
-      <c r="M4">
+      <c r="L4" s="4">
+        <f>MIN(C4*'historicals_input'!$B29,C4)</f>
+        <v/>
+      </c>
+      <c r="M4" s="4">
         <f>MIN(MAX(K4-L4-'historicals_input'!$B19,0),E4)</f>
         <v/>
       </c>
-      <c r="N4">
-        <f>MIN(MAX(K4-L4-M4-'historicals_input'!$B19,0),MAX(C4-L4,0))</f>
-        <v/>
-      </c>
-      <c r="O4">
-        <f>MIN(MAX(K4-L4-M4-N4-'historicals_input'!$B19,0),D4+I4)</f>
-        <v/>
-      </c>
-      <c r="P4">
-        <f>MAX('historicals_input'!$B19-(K4-L4-M4-N4-O4),0)</f>
-        <v/>
-      </c>
-      <c r="Q4">
-        <f>K4-L4-M4-N4-O4+P4</f>
-        <v/>
-      </c>
-      <c r="R4">
-        <f>MAX(C4-L4-N4,0)</f>
-        <v/>
-      </c>
-      <c r="S4">
-        <f>MAX(D4+I4-O4,0)</f>
-        <v/>
-      </c>
-      <c r="T4">
-        <f>MAX(E4-M4+P4,0)</f>
+      <c r="N4" s="4">
+        <f>K4-L4-M4</f>
+        <v/>
+      </c>
+      <c r="O4" s="4">
+        <f>MAX(N4-'historicals_input'!$B19,0)*'historicals_input'!$B30</f>
+        <v/>
+      </c>
+      <c r="P4" s="4">
+        <f>MIN(O4,MAX(C4-L4,0))</f>
+        <v/>
+      </c>
+      <c r="Q4" s="4">
+        <f>MIN(MAX(O4-P4,0),D4+I4)</f>
+        <v/>
+      </c>
+      <c r="R4" s="4">
+        <f>MIN(MAX('historicals_input'!$B19-(N4-P4-Q4),0),MAX('historicals_input'!$B28-E4+M4,0))</f>
+        <v/>
+      </c>
+      <c r="S4" s="4">
+        <f>MAX('historicals_input'!$B19-(N4-P4-Q4-R4),0)</f>
+        <v/>
+      </c>
+      <c r="T4" s="4">
+        <f>N4-P4-Q4+R4</f>
+        <v/>
+      </c>
+      <c r="U4" s="4">
+        <f>MAX(C4-L4-P4,0)</f>
+        <v/>
+      </c>
+      <c r="V4" s="4">
+        <f>MAX(D4+I4-Q4,0)</f>
+        <v/>
+      </c>
+      <c r="W4" s="4">
+        <f>MAX(E4-M4+R4,0)</f>
         <v/>
       </c>
     </row>
@@ -2365,80 +2445,92 @@
       <c r="A5" t="n">
         <v>2026</v>
       </c>
-      <c r="B5">
-        <f>Q4</f>
-        <v/>
-      </c>
-      <c r="C5">
-        <f>R4</f>
-        <v/>
-      </c>
-      <c r="D5">
-        <f>S4</f>
-        <v/>
-      </c>
-      <c r="E5">
+      <c r="B5" s="4">
         <f>T4</f>
         <v/>
       </c>
-      <c r="F5">
+      <c r="C5" s="4">
+        <f>U4</f>
+        <v/>
+      </c>
+      <c r="D5" s="4">
+        <f>V4</f>
+        <v/>
+      </c>
+      <c r="E5" s="4">
+        <f>W4</f>
+        <v/>
+      </c>
+      <c r="F5" s="4">
         <f>'operating_model'!$C17</f>
         <v/>
       </c>
-      <c r="G5">
+      <c r="G5" s="4">
         <f>C5*'historicals_input'!$B24</f>
         <v/>
       </c>
-      <c r="H5">
+      <c r="H5" s="4">
         <f>D5*'historicals_input'!$B25</f>
         <v/>
       </c>
-      <c r="I5">
+      <c r="I5" s="4">
         <f>D5*'historicals_input'!$B26</f>
         <v/>
       </c>
-      <c r="J5">
+      <c r="J5" s="4">
         <f>E5*'historicals_input'!$B27</f>
         <v/>
       </c>
-      <c r="K5">
+      <c r="K5" s="4">
         <f>B5+F5-G5-H5-J5</f>
         <v/>
       </c>
-      <c r="L5">
-        <f>MIN(C5*'historicals_input'!$B28,C5)</f>
-        <v/>
-      </c>
-      <c r="M5">
+      <c r="L5" s="4">
+        <f>MIN(C5*'historicals_input'!$B29,C5)</f>
+        <v/>
+      </c>
+      <c r="M5" s="4">
         <f>MIN(MAX(K5-L5-'historicals_input'!$B19,0),E5)</f>
         <v/>
       </c>
-      <c r="N5">
-        <f>MIN(MAX(K5-L5-M5-'historicals_input'!$B19,0),MAX(C5-L5,0))</f>
-        <v/>
-      </c>
-      <c r="O5">
-        <f>MIN(MAX(K5-L5-M5-N5-'historicals_input'!$B19,0),D5+I5)</f>
-        <v/>
-      </c>
-      <c r="P5">
-        <f>MAX('historicals_input'!$B19-(K5-L5-M5-N5-O5),0)</f>
-        <v/>
-      </c>
-      <c r="Q5">
-        <f>K5-L5-M5-N5-O5+P5</f>
-        <v/>
-      </c>
-      <c r="R5">
-        <f>MAX(C5-L5-N5,0)</f>
-        <v/>
-      </c>
-      <c r="S5">
-        <f>MAX(D5+I5-O5,0)</f>
-        <v/>
-      </c>
-      <c r="T5">
-        <f>MAX(E5-M5+P5,0)</f>
+      <c r="N5" s="4">
+        <f>K5-L5-M5</f>
+        <v/>
+      </c>
+      <c r="O5" s="4">
+        <f>MAX(N5-'historicals_input'!$B19,0)*'historicals_input'!$B30</f>
+        <v/>
+      </c>
+      <c r="P5" s="4">
+        <f>MIN(O5,MAX(C5-L5,0))</f>
+        <v/>
+      </c>
+      <c r="Q5" s="4">
+        <f>MIN(MAX(O5-P5,0),D5+I5)</f>
+        <v/>
+      </c>
+      <c r="R5" s="4">
+        <f>MIN(MAX('historicals_input'!$B19-(N5-P5-Q5),0),MAX('historicals_input'!$B28-E5+M5,0))</f>
+        <v/>
+      </c>
+      <c r="S5" s="4">
+        <f>MAX('historicals_input'!$B19-(N5-P5-Q5-R5),0)</f>
+        <v/>
+      </c>
+      <c r="T5" s="4">
+        <f>N5-P5-Q5+R5</f>
+        <v/>
+      </c>
+      <c r="U5" s="4">
+        <f>MAX(C5-L5-P5,0)</f>
+        <v/>
+      </c>
+      <c r="V5" s="4">
+        <f>MAX(D5+I5-Q5,0)</f>
+        <v/>
+      </c>
+      <c r="W5" s="4">
+        <f>MAX(E5-M5+R5,0)</f>
         <v/>
       </c>
     </row>
@@ -2446,80 +2538,92 @@
       <c r="A6" t="n">
         <v>2027</v>
       </c>
-      <c r="B6">
-        <f>Q5</f>
-        <v/>
-      </c>
-      <c r="C6">
-        <f>R5</f>
-        <v/>
-      </c>
-      <c r="D6">
-        <f>S5</f>
-        <v/>
-      </c>
-      <c r="E6">
+      <c r="B6" s="4">
         <f>T5</f>
         <v/>
       </c>
-      <c r="F6">
+      <c r="C6" s="4">
+        <f>U5</f>
+        <v/>
+      </c>
+      <c r="D6" s="4">
+        <f>V5</f>
+        <v/>
+      </c>
+      <c r="E6" s="4">
+        <f>W5</f>
+        <v/>
+      </c>
+      <c r="F6" s="4">
         <f>'operating_model'!$D17</f>
         <v/>
       </c>
-      <c r="G6">
+      <c r="G6" s="4">
         <f>C6*'historicals_input'!$B24</f>
         <v/>
       </c>
-      <c r="H6">
+      <c r="H6" s="4">
         <f>D6*'historicals_input'!$B25</f>
         <v/>
       </c>
-      <c r="I6">
+      <c r="I6" s="4">
         <f>D6*'historicals_input'!$B26</f>
         <v/>
       </c>
-      <c r="J6">
+      <c r="J6" s="4">
         <f>E6*'historicals_input'!$B27</f>
         <v/>
       </c>
-      <c r="K6">
+      <c r="K6" s="4">
         <f>B6+F6-G6-H6-J6</f>
         <v/>
       </c>
-      <c r="L6">
-        <f>MIN(C6*'historicals_input'!$B28,C6)</f>
-        <v/>
-      </c>
-      <c r="M6">
+      <c r="L6" s="4">
+        <f>MIN(C6*'historicals_input'!$B29,C6)</f>
+        <v/>
+      </c>
+      <c r="M6" s="4">
         <f>MIN(MAX(K6-L6-'historicals_input'!$B19,0),E6)</f>
         <v/>
       </c>
-      <c r="N6">
-        <f>MIN(MAX(K6-L6-M6-'historicals_input'!$B19,0),MAX(C6-L6,0))</f>
-        <v/>
-      </c>
-      <c r="O6">
-        <f>MIN(MAX(K6-L6-M6-N6-'historicals_input'!$B19,0),D6+I6)</f>
-        <v/>
-      </c>
-      <c r="P6">
-        <f>MAX('historicals_input'!$B19-(K6-L6-M6-N6-O6),0)</f>
-        <v/>
-      </c>
-      <c r="Q6">
-        <f>K6-L6-M6-N6-O6+P6</f>
-        <v/>
-      </c>
-      <c r="R6">
-        <f>MAX(C6-L6-N6,0)</f>
-        <v/>
-      </c>
-      <c r="S6">
-        <f>MAX(D6+I6-O6,0)</f>
-        <v/>
-      </c>
-      <c r="T6">
-        <f>MAX(E6-M6+P6,0)</f>
+      <c r="N6" s="4">
+        <f>K6-L6-M6</f>
+        <v/>
+      </c>
+      <c r="O6" s="4">
+        <f>MAX(N6-'historicals_input'!$B19,0)*'historicals_input'!$B30</f>
+        <v/>
+      </c>
+      <c r="P6" s="4">
+        <f>MIN(O6,MAX(C6-L6,0))</f>
+        <v/>
+      </c>
+      <c r="Q6" s="4">
+        <f>MIN(MAX(O6-P6,0),D6+I6)</f>
+        <v/>
+      </c>
+      <c r="R6" s="4">
+        <f>MIN(MAX('historicals_input'!$B19-(N6-P6-Q6),0),MAX('historicals_input'!$B28-E6+M6,0))</f>
+        <v/>
+      </c>
+      <c r="S6" s="4">
+        <f>MAX('historicals_input'!$B19-(N6-P6-Q6-R6),0)</f>
+        <v/>
+      </c>
+      <c r="T6" s="4">
+        <f>N6-P6-Q6+R6</f>
+        <v/>
+      </c>
+      <c r="U6" s="4">
+        <f>MAX(C6-L6-P6,0)</f>
+        <v/>
+      </c>
+      <c r="V6" s="4">
+        <f>MAX(D6+I6-Q6,0)</f>
+        <v/>
+      </c>
+      <c r="W6" s="4">
+        <f>MAX(E6-M6+R6,0)</f>
         <v/>
       </c>
     </row>
@@ -2527,80 +2631,92 @@
       <c r="A7" t="n">
         <v>2028</v>
       </c>
-      <c r="B7">
-        <f>Q6</f>
-        <v/>
-      </c>
-      <c r="C7">
-        <f>R6</f>
-        <v/>
-      </c>
-      <c r="D7">
-        <f>S6</f>
-        <v/>
-      </c>
-      <c r="E7">
+      <c r="B7" s="4">
         <f>T6</f>
         <v/>
       </c>
-      <c r="F7">
+      <c r="C7" s="4">
+        <f>U6</f>
+        <v/>
+      </c>
+      <c r="D7" s="4">
+        <f>V6</f>
+        <v/>
+      </c>
+      <c r="E7" s="4">
+        <f>W6</f>
+        <v/>
+      </c>
+      <c r="F7" s="4">
         <f>'operating_model'!$E17</f>
         <v/>
       </c>
-      <c r="G7">
+      <c r="G7" s="4">
         <f>C7*'historicals_input'!$B24</f>
         <v/>
       </c>
-      <c r="H7">
+      <c r="H7" s="4">
         <f>D7*'historicals_input'!$B25</f>
         <v/>
       </c>
-      <c r="I7">
+      <c r="I7" s="4">
         <f>D7*'historicals_input'!$B26</f>
         <v/>
       </c>
-      <c r="J7">
+      <c r="J7" s="4">
         <f>E7*'historicals_input'!$B27</f>
         <v/>
       </c>
-      <c r="K7">
+      <c r="K7" s="4">
         <f>B7+F7-G7-H7-J7</f>
         <v/>
       </c>
-      <c r="L7">
-        <f>MIN(C7*'historicals_input'!$B28,C7)</f>
-        <v/>
-      </c>
-      <c r="M7">
+      <c r="L7" s="4">
+        <f>MIN(C7*'historicals_input'!$B29,C7)</f>
+        <v/>
+      </c>
+      <c r="M7" s="4">
         <f>MIN(MAX(K7-L7-'historicals_input'!$B19,0),E7)</f>
         <v/>
       </c>
-      <c r="N7">
-        <f>MIN(MAX(K7-L7-M7-'historicals_input'!$B19,0),MAX(C7-L7,0))</f>
-        <v/>
-      </c>
-      <c r="O7">
-        <f>MIN(MAX(K7-L7-M7-N7-'historicals_input'!$B19,0),D7+I7)</f>
-        <v/>
-      </c>
-      <c r="P7">
-        <f>MAX('historicals_input'!$B19-(K7-L7-M7-N7-O7),0)</f>
-        <v/>
-      </c>
-      <c r="Q7">
-        <f>K7-L7-M7-N7-O7+P7</f>
-        <v/>
-      </c>
-      <c r="R7">
-        <f>MAX(C7-L7-N7,0)</f>
-        <v/>
-      </c>
-      <c r="S7">
-        <f>MAX(D7+I7-O7,0)</f>
-        <v/>
-      </c>
-      <c r="T7">
-        <f>MAX(E7-M7+P7,0)</f>
+      <c r="N7" s="4">
+        <f>K7-L7-M7</f>
+        <v/>
+      </c>
+      <c r="O7" s="4">
+        <f>MAX(N7-'historicals_input'!$B19,0)*'historicals_input'!$B30</f>
+        <v/>
+      </c>
+      <c r="P7" s="4">
+        <f>MIN(O7,MAX(C7-L7,0))</f>
+        <v/>
+      </c>
+      <c r="Q7" s="4">
+        <f>MIN(MAX(O7-P7,0),D7+I7)</f>
+        <v/>
+      </c>
+      <c r="R7" s="4">
+        <f>MIN(MAX('historicals_input'!$B19-(N7-P7-Q7),0),MAX('historicals_input'!$B28-E7+M7,0))</f>
+        <v/>
+      </c>
+      <c r="S7" s="4">
+        <f>MAX('historicals_input'!$B19-(N7-P7-Q7-R7),0)</f>
+        <v/>
+      </c>
+      <c r="T7" s="4">
+        <f>N7-P7-Q7+R7</f>
+        <v/>
+      </c>
+      <c r="U7" s="4">
+        <f>MAX(C7-L7-P7,0)</f>
+        <v/>
+      </c>
+      <c r="V7" s="4">
+        <f>MAX(D7+I7-Q7,0)</f>
+        <v/>
+      </c>
+      <c r="W7" s="4">
+        <f>MAX(E7-M7+R7,0)</f>
         <v/>
       </c>
     </row>
@@ -2608,80 +2724,92 @@
       <c r="A8" t="n">
         <v>2029</v>
       </c>
-      <c r="B8">
-        <f>Q7</f>
-        <v/>
-      </c>
-      <c r="C8">
-        <f>R7</f>
-        <v/>
-      </c>
-      <c r="D8">
-        <f>S7</f>
-        <v/>
-      </c>
-      <c r="E8">
+      <c r="B8" s="4">
         <f>T7</f>
         <v/>
       </c>
-      <c r="F8">
+      <c r="C8" s="4">
+        <f>U7</f>
+        <v/>
+      </c>
+      <c r="D8" s="4">
+        <f>V7</f>
+        <v/>
+      </c>
+      <c r="E8" s="4">
+        <f>W7</f>
+        <v/>
+      </c>
+      <c r="F8" s="4">
         <f>'operating_model'!$F17</f>
         <v/>
       </c>
-      <c r="G8">
+      <c r="G8" s="4">
         <f>C8*'historicals_input'!$B24</f>
         <v/>
       </c>
-      <c r="H8">
+      <c r="H8" s="4">
         <f>D8*'historicals_input'!$B25</f>
         <v/>
       </c>
-      <c r="I8">
+      <c r="I8" s="4">
         <f>D8*'historicals_input'!$B26</f>
         <v/>
       </c>
-      <c r="J8">
+      <c r="J8" s="4">
         <f>E8*'historicals_input'!$B27</f>
         <v/>
       </c>
-      <c r="K8">
+      <c r="K8" s="4">
         <f>B8+F8-G8-H8-J8</f>
         <v/>
       </c>
-      <c r="L8">
-        <f>MIN(C8*'historicals_input'!$B28,C8)</f>
-        <v/>
-      </c>
-      <c r="M8">
+      <c r="L8" s="4">
+        <f>MIN(C8*'historicals_input'!$B29,C8)</f>
+        <v/>
+      </c>
+      <c r="M8" s="4">
         <f>MIN(MAX(K8-L8-'historicals_input'!$B19,0),E8)</f>
         <v/>
       </c>
-      <c r="N8">
-        <f>MIN(MAX(K8-L8-M8-'historicals_input'!$B19,0),MAX(C8-L8,0))</f>
-        <v/>
-      </c>
-      <c r="O8">
-        <f>MIN(MAX(K8-L8-M8-N8-'historicals_input'!$B19,0),D8+I8)</f>
-        <v/>
-      </c>
-      <c r="P8">
-        <f>MAX('historicals_input'!$B19-(K8-L8-M8-N8-O8),0)</f>
-        <v/>
-      </c>
-      <c r="Q8">
-        <f>K8-L8-M8-N8-O8+P8</f>
-        <v/>
-      </c>
-      <c r="R8">
-        <f>MAX(C8-L8-N8,0)</f>
-        <v/>
-      </c>
-      <c r="S8">
-        <f>MAX(D8+I8-O8,0)</f>
-        <v/>
-      </c>
-      <c r="T8">
-        <f>MAX(E8-M8+P8,0)</f>
+      <c r="N8" s="4">
+        <f>K8-L8-M8</f>
+        <v/>
+      </c>
+      <c r="O8" s="4">
+        <f>MAX(N8-'historicals_input'!$B19,0)*'historicals_input'!$B30</f>
+        <v/>
+      </c>
+      <c r="P8" s="4">
+        <f>MIN(O8,MAX(C8-L8,0))</f>
+        <v/>
+      </c>
+      <c r="Q8" s="4">
+        <f>MIN(MAX(O8-P8,0),D8+I8)</f>
+        <v/>
+      </c>
+      <c r="R8" s="4">
+        <f>MIN(MAX('historicals_input'!$B19-(N8-P8-Q8),0),MAX('historicals_input'!$B28-E8+M8,0))</f>
+        <v/>
+      </c>
+      <c r="S8" s="4">
+        <f>MAX('historicals_input'!$B19-(N8-P8-Q8-R8),0)</f>
+        <v/>
+      </c>
+      <c r="T8" s="4">
+        <f>N8-P8-Q8+R8</f>
+        <v/>
+      </c>
+      <c r="U8" s="4">
+        <f>MAX(C8-L8-P8,0)</f>
+        <v/>
+      </c>
+      <c r="V8" s="4">
+        <f>MAX(D8+I8-Q8,0)</f>
+        <v/>
+      </c>
+      <c r="W8" s="4">
+        <f>MAX(E8-M8+R8,0)</f>
         <v/>
       </c>
     </row>
@@ -2696,10 +2824,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -2737,121 +2865,220 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sponsor Equity</t>
+          <t>Entry Senior Debt</t>
         </is>
       </c>
       <c r="B5" s="4">
-        <f>'sources_uses'!$B17</f>
+        <f>'sources_uses'!$B14</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Exit EBITDA</t>
+          <t>Entry Sub Debt</t>
         </is>
       </c>
       <c r="B6" s="4">
-        <f>'operating_model'!$F7</f>
+        <f>'sources_uses'!$B15</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Exit Multiple</t>
+          <t>Entry Net Debt</t>
         </is>
       </c>
       <c r="B7" s="4">
-        <f>'historicals_input'!$B37</f>
+        <f>B5+B6</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Exit EV</t>
+          <t>Sponsor Equity</t>
         </is>
       </c>
       <c r="B8" s="4">
-        <f>B6*B7</f>
+        <f>'sources_uses'!$B17</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Exit Senior Debt</t>
-        </is>
-      </c>
-      <c r="B9" s="4">
-        <f>'debt_schedule'!$R8</f>
+          <t>Entry Debt / EBITDA</t>
+        </is>
+      </c>
+      <c r="B9" s="8">
+        <f>IFERROR(B7/'historicals_input'!$B13,0)</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Exit Sub Debt</t>
+          <t>Exit EBITDA</t>
         </is>
       </c>
       <c r="B10" s="4">
-        <f>'debt_schedule'!$S8</f>
+        <f>'operating_model'!$F7</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Exit Revolver</t>
-        </is>
-      </c>
-      <c r="B11" s="4">
-        <f>'debt_schedule'!$T8</f>
+          <t>Exit Multiple</t>
+        </is>
+      </c>
+      <c r="B11" s="6">
+        <f>'historicals_input'!$B39</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Exit Cash</t>
+          <t>Exit EV</t>
         </is>
       </c>
       <c r="B12" s="4">
-        <f>'debt_schedule'!$Q8</f>
+        <f>B10*B11</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Exit Equity Value</t>
+          <t>Exit Senior Debt</t>
         </is>
       </c>
       <c r="B13" s="4">
-        <f>B8-B9-B10-B11+B12</f>
+        <f>'debt_schedule'!$U8</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MOIC</t>
-        </is>
-      </c>
-      <c r="B14" s="8">
-        <f>IFERROR(B13/B5,0)</f>
+          <t>Exit Sub Debt</t>
+        </is>
+      </c>
+      <c r="B14" s="4">
+        <f>'debt_schedule'!$V8</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>Exit Revolver</t>
+        </is>
+      </c>
+      <c r="B15" s="4">
+        <f>'debt_schedule'!$W8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Exit Cash</t>
+        </is>
+      </c>
+      <c r="B16" s="4">
+        <f>'debt_schedule'!$T8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Exit Net Debt</t>
+        </is>
+      </c>
+      <c r="B17" s="4">
+        <f>B13+B14+B15-B16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Exit Debt / EBITDA</t>
+        </is>
+      </c>
+      <c r="B18" s="8">
+        <f>IFERROR(B17/B10,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Debt Paydown</t>
+        </is>
+      </c>
+      <c r="B19" s="4">
+        <f>B7-B17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Exit Equity Value</t>
+        </is>
+      </c>
+      <c r="B20" s="4">
+        <f>B12-B13-B14-B15+B16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>MOIC</t>
+        </is>
+      </c>
+      <c r="B21" s="8">
+        <f>IFERROR(B20/B8,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>IRR</t>
         </is>
       </c>
-      <c r="B15" s="5">
-        <f>IFERROR(B14^(1/5)-1,0)</f>
+      <c r="B22" s="5">
+        <f>IFERROR(B21^(1/5)-1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Revenue CAGR</t>
+        </is>
+      </c>
+      <c r="B23" s="5">
+        <f>IFERROR((operating_model!F4/historicals_input!B7)^(1/5)-1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>EBITDA CAGR</t>
+        </is>
+      </c>
+      <c r="B24" s="5">
+        <f>IFERROR((B10/historicals_input!C7)^(1/5)-1,0)</f>
         <v/>
       </c>
     </row>
@@ -2955,7 +3182,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>'historicals_input'!$B32</f>
+        <f>'historicals_input'!$B34</f>
         <v/>
       </c>
       <c r="D5" t="inlineStr">
@@ -2991,7 +3218,7 @@
         </is>
       </c>
       <c r="B6" s="7">
-        <f>'historicals_input'!$B33</f>
+        <f>'historicals_input'!$B35</f>
         <v/>
       </c>
       <c r="D6" t="inlineStr">
@@ -3027,7 +3254,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>'historicals_input'!$B34</f>
+        <f>'historicals_input'!$B36</f>
         <v/>
       </c>
       <c r="D7" t="inlineStr">
@@ -3074,7 +3301,7 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>'historicals_input'!$B35</f>
+        <f>'historicals_input'!$B37</f>
         <v/>
       </c>
       <c r="D9" t="inlineStr">
@@ -3083,7 +3310,7 @@
         </is>
       </c>
       <c r="E9">
-        <f>'historicals_input'!$B36</f>
+        <f>'historicals_input'!$B38</f>
         <v/>
       </c>
     </row>
@@ -3094,7 +3321,7 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>'historicals_input'!$B31</f>
+        <f>'historicals_input'!$B33</f>
         <v/>
       </c>
       <c r="D10" t="inlineStr">
@@ -3103,7 +3330,7 @@
         </is>
       </c>
       <c r="E10">
-        <f>'historicals_input'!$B37</f>
+        <f>'historicals_input'!$B39</f>
         <v/>
       </c>
     </row>
@@ -3134,7 +3361,7 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>'returns'!$B5/('returns'!$B5+'sources_uses'!$B14+'sources_uses'!$B15)</f>
+        <f>'returns'!$B8/('returns'!$B8+'sources_uses'!$B14+'sources_uses'!$B15)</f>
         <v/>
       </c>
       <c r="D12" t="inlineStr">
@@ -3227,7 +3454,7 @@
         </is>
       </c>
       <c r="E18" s="4">
-        <f>E16-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8</f>
+        <f>E16-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8</f>
         <v/>
       </c>
     </row>
@@ -3238,7 +3465,7 @@
         </is>
       </c>
       <c r="E19" s="4">
-        <f>E17-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8</f>
+        <f>E17-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8</f>
         <v/>
       </c>
     </row>
@@ -3329,23 +3556,23 @@
         <v>0.104</v>
       </c>
       <c r="B6" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A6)^{1,2,3,4,5})+((valuation!I5*(1+B5))/MAX(A6-B5,0.0001))/(1+A6)^5-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'historicals_input'!$B12</f>
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A6)^{1,2,3,4,5})+((valuation!I5*(1+B5))/MAX(A6-B5,0.0001))/(1+A6)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
         <v/>
       </c>
       <c r="C6" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A6)^{1,2,3,4,5})+((valuation!I5*(1+C5))/MAX(A6-C5,0.0001))/(1+A6)^5-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'historicals_input'!$B12</f>
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A6)^{1,2,3,4,5})+((valuation!I5*(1+C5))/MAX(A6-C5,0.0001))/(1+A6)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
         <v/>
       </c>
       <c r="D6" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A6)^{1,2,3,4,5})+((valuation!I5*(1+D5))/MAX(A6-D5,0.0001))/(1+A6)^5-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'historicals_input'!$B12</f>
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A6)^{1,2,3,4,5})+((valuation!I5*(1+D5))/MAX(A6-D5,0.0001))/(1+A6)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
         <v/>
       </c>
       <c r="E6" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A6)^{1,2,3,4,5})+((valuation!I5*(1+E5))/MAX(A6-E5,0.0001))/(1+A6)^5-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'historicals_input'!$B12</f>
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A6)^{1,2,3,4,5})+((valuation!I5*(1+E5))/MAX(A6-E5,0.0001))/(1+A6)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
         <v/>
       </c>
       <c r="F6" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A6)^{1,2,3,4,5})+((valuation!I5*(1+F5))/MAX(A6-F5,0.0001))/(1+A6)^5-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'historicals_input'!$B12</f>
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A6)^{1,2,3,4,5})+((valuation!I5*(1+F5))/MAX(A6-F5,0.0001))/(1+A6)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
         <v/>
       </c>
     </row>
@@ -3354,23 +3581,23 @@
         <v>0.109</v>
       </c>
       <c r="B7" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A7)^{1,2,3,4,5})+((valuation!I5*(1+B5))/MAX(A7-B5,0.0001))/(1+A7)^5-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'historicals_input'!$B12</f>
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A7)^{1,2,3,4,5})+((valuation!I5*(1+B5))/MAX(A7-B5,0.0001))/(1+A7)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
         <v/>
       </c>
       <c r="C7" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A7)^{1,2,3,4,5})+((valuation!I5*(1+C5))/MAX(A7-C5,0.0001))/(1+A7)^5-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'historicals_input'!$B12</f>
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A7)^{1,2,3,4,5})+((valuation!I5*(1+C5))/MAX(A7-C5,0.0001))/(1+A7)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
         <v/>
       </c>
       <c r="D7" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A7)^{1,2,3,4,5})+((valuation!I5*(1+D5))/MAX(A7-D5,0.0001))/(1+A7)^5-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'historicals_input'!$B12</f>
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A7)^{1,2,3,4,5})+((valuation!I5*(1+D5))/MAX(A7-D5,0.0001))/(1+A7)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
         <v/>
       </c>
       <c r="E7" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A7)^{1,2,3,4,5})+((valuation!I5*(1+E5))/MAX(A7-E5,0.0001))/(1+A7)^5-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'historicals_input'!$B12</f>
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A7)^{1,2,3,4,5})+((valuation!I5*(1+E5))/MAX(A7-E5,0.0001))/(1+A7)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
         <v/>
       </c>
       <c r="F7" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A7)^{1,2,3,4,5})+((valuation!I5*(1+F5))/MAX(A7-F5,0.0001))/(1+A7)^5-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'historicals_input'!$B12</f>
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A7)^{1,2,3,4,5})+((valuation!I5*(1+F5))/MAX(A7-F5,0.0001))/(1+A7)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
         <v/>
       </c>
     </row>
@@ -3379,23 +3606,23 @@
         <v>0.114</v>
       </c>
       <c r="B8" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A8)^{1,2,3,4,5})+((valuation!I5*(1+B5))/MAX(A8-B5,0.0001))/(1+A8)^5-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'historicals_input'!$B12</f>
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A8)^{1,2,3,4,5})+((valuation!I5*(1+B5))/MAX(A8-B5,0.0001))/(1+A8)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
         <v/>
       </c>
       <c r="C8" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A8)^{1,2,3,4,5})+((valuation!I5*(1+C5))/MAX(A8-C5,0.0001))/(1+A8)^5-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'historicals_input'!$B12</f>
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A8)^{1,2,3,4,5})+((valuation!I5*(1+C5))/MAX(A8-C5,0.0001))/(1+A8)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
         <v/>
       </c>
       <c r="D8" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A8)^{1,2,3,4,5})+((valuation!I5*(1+D5))/MAX(A8-D5,0.0001))/(1+A8)^5-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'historicals_input'!$B12</f>
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A8)^{1,2,3,4,5})+((valuation!I5*(1+D5))/MAX(A8-D5,0.0001))/(1+A8)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
         <v/>
       </c>
       <c r="E8" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A8)^{1,2,3,4,5})+((valuation!I5*(1+E5))/MAX(A8-E5,0.0001))/(1+A8)^5-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'historicals_input'!$B12</f>
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A8)^{1,2,3,4,5})+((valuation!I5*(1+E5))/MAX(A8-E5,0.0001))/(1+A8)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
         <v/>
       </c>
       <c r="F8" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A8)^{1,2,3,4,5})+((valuation!I5*(1+F5))/MAX(A8-F5,0.0001))/(1+A8)^5-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'historicals_input'!$B12</f>
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A8)^{1,2,3,4,5})+((valuation!I5*(1+F5))/MAX(A8-F5,0.0001))/(1+A8)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
         <v/>
       </c>
     </row>
@@ -3404,23 +3631,23 @@
         <v>0.119</v>
       </c>
       <c r="B9" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A9)^{1,2,3,4,5})+((valuation!I5*(1+B5))/MAX(A9-B5,0.0001))/(1+A9)^5-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'historicals_input'!$B12</f>
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A9)^{1,2,3,4,5})+((valuation!I5*(1+B5))/MAX(A9-B5,0.0001))/(1+A9)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
         <v/>
       </c>
       <c r="C9" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A9)^{1,2,3,4,5})+((valuation!I5*(1+C5))/MAX(A9-C5,0.0001))/(1+A9)^5-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'historicals_input'!$B12</f>
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A9)^{1,2,3,4,5})+((valuation!I5*(1+C5))/MAX(A9-C5,0.0001))/(1+A9)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
         <v/>
       </c>
       <c r="D9" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A9)^{1,2,3,4,5})+((valuation!I5*(1+D5))/MAX(A9-D5,0.0001))/(1+A9)^5-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'historicals_input'!$B12</f>
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A9)^{1,2,3,4,5})+((valuation!I5*(1+D5))/MAX(A9-D5,0.0001))/(1+A9)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
         <v/>
       </c>
       <c r="E9" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A9)^{1,2,3,4,5})+((valuation!I5*(1+E5))/MAX(A9-E5,0.0001))/(1+A9)^5-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'historicals_input'!$B12</f>
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A9)^{1,2,3,4,5})+((valuation!I5*(1+E5))/MAX(A9-E5,0.0001))/(1+A9)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
         <v/>
       </c>
       <c r="F9" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A9)^{1,2,3,4,5})+((valuation!I5*(1+F5))/MAX(A9-F5,0.0001))/(1+A9)^5-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'historicals_input'!$B12</f>
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A9)^{1,2,3,4,5})+((valuation!I5*(1+F5))/MAX(A9-F5,0.0001))/(1+A9)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
         <v/>
       </c>
     </row>
@@ -3429,23 +3656,23 @@
         <v>0.124</v>
       </c>
       <c r="B10" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A10)^{1,2,3,4,5})+((valuation!I5*(1+B5))/MAX(A10-B5,0.0001))/(1+A10)^5-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'historicals_input'!$B12</f>
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A10)^{1,2,3,4,5})+((valuation!I5*(1+B5))/MAX(A10-B5,0.0001))/(1+A10)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A10)^{1,2,3,4,5})+((valuation!I5*(1+C5))/MAX(A10-C5,0.0001))/(1+A10)^5-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'historicals_input'!$B12</f>
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A10)^{1,2,3,4,5})+((valuation!I5*(1+C5))/MAX(A10-C5,0.0001))/(1+A10)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
         <v/>
       </c>
       <c r="D10" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A10)^{1,2,3,4,5})+((valuation!I5*(1+D5))/MAX(A10-D5,0.0001))/(1+A10)^5-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'historicals_input'!$B12</f>
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A10)^{1,2,3,4,5})+((valuation!I5*(1+D5))/MAX(A10-D5,0.0001))/(1+A10)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
         <v/>
       </c>
       <c r="E10" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A10)^{1,2,3,4,5})+((valuation!I5*(1+E5))/MAX(A10-E5,0.0001))/(1+A10)^5-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'historicals_input'!$B12</f>
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A10)^{1,2,3,4,5})+((valuation!I5*(1+E5))/MAX(A10-E5,0.0001))/(1+A10)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
         <v/>
       </c>
       <c r="F10" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A10)^{1,2,3,4,5})+((valuation!I5*(1+F5))/MAX(A10-F5,0.0001))/(1+A10)^5-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'historicals_input'!$B12</f>
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A10)^{1,2,3,4,5})+((valuation!I5*(1+F5))/MAX(A10-F5,0.0001))/(1+A10)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
         <v/>
       </c>
     </row>
@@ -3486,23 +3713,23 @@
         <v>9</v>
       </c>
       <c r="B16" s="8">
-        <f>((('returns'!$B6*(1+B15))*A16)-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'returns'!$B5</f>
+        <f>((('returns'!$B10*(1+B15))*A16)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
         <v/>
       </c>
       <c r="C16" s="8">
-        <f>((('returns'!$B6*(1+C15))*A16)-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'returns'!$B5</f>
+        <f>((('returns'!$B10*(1+C15))*A16)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
         <v/>
       </c>
       <c r="D16" s="8">
-        <f>((('returns'!$B6*(1+D15))*A16)-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'returns'!$B5</f>
+        <f>((('returns'!$B10*(1+D15))*A16)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
         <v/>
       </c>
       <c r="E16" s="8">
-        <f>((('returns'!$B6*(1+E15))*A16)-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'returns'!$B5</f>
+        <f>((('returns'!$B10*(1+E15))*A16)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
         <v/>
       </c>
       <c r="F16" s="8">
-        <f>((('returns'!$B6*(1+F15))*A16)-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'returns'!$B5</f>
+        <f>((('returns'!$B10*(1+F15))*A16)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
         <v/>
       </c>
     </row>
@@ -3511,23 +3738,23 @@
         <v>9.5</v>
       </c>
       <c r="B17" s="8">
-        <f>((('returns'!$B6*(1+B15))*A17)-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'returns'!$B5</f>
+        <f>((('returns'!$B10*(1+B15))*A17)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
         <v/>
       </c>
       <c r="C17" s="8">
-        <f>((('returns'!$B6*(1+C15))*A17)-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'returns'!$B5</f>
+        <f>((('returns'!$B10*(1+C15))*A17)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>((('returns'!$B6*(1+D15))*A17)-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'returns'!$B5</f>
+        <f>((('returns'!$B10*(1+D15))*A17)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
         <v/>
       </c>
       <c r="E17" s="8">
-        <f>((('returns'!$B6*(1+E15))*A17)-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'returns'!$B5</f>
+        <f>((('returns'!$B10*(1+E15))*A17)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
         <v/>
       </c>
       <c r="F17" s="8">
-        <f>((('returns'!$B6*(1+F15))*A17)-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'returns'!$B5</f>
+        <f>((('returns'!$B10*(1+F15))*A17)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
         <v/>
       </c>
     </row>
@@ -3536,23 +3763,23 @@
         <v>10</v>
       </c>
       <c r="B18" s="8">
-        <f>((('returns'!$B6*(1+B15))*A18)-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'returns'!$B5</f>
+        <f>((('returns'!$B10*(1+B15))*A18)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
         <v/>
       </c>
       <c r="C18" s="8">
-        <f>((('returns'!$B6*(1+C15))*A18)-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'returns'!$B5</f>
+        <f>((('returns'!$B10*(1+C15))*A18)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
         <v/>
       </c>
       <c r="D18" s="8">
-        <f>((('returns'!$B6*(1+D15))*A18)-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'returns'!$B5</f>
+        <f>((('returns'!$B10*(1+D15))*A18)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
         <v/>
       </c>
       <c r="E18" s="8">
-        <f>((('returns'!$B6*(1+E15))*A18)-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'returns'!$B5</f>
+        <f>((('returns'!$B10*(1+E15))*A18)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
         <v/>
       </c>
       <c r="F18" s="8">
-        <f>((('returns'!$B6*(1+F15))*A18)-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'returns'!$B5</f>
+        <f>((('returns'!$B10*(1+F15))*A18)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
         <v/>
       </c>
     </row>
@@ -3561,23 +3788,23 @@
         <v>10.5</v>
       </c>
       <c r="B19" s="8">
-        <f>((('returns'!$B6*(1+B15))*A19)-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'returns'!$B5</f>
+        <f>((('returns'!$B10*(1+B15))*A19)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
         <v/>
       </c>
       <c r="C19" s="8">
-        <f>((('returns'!$B6*(1+C15))*A19)-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'returns'!$B5</f>
+        <f>((('returns'!$B10*(1+C15))*A19)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
         <v/>
       </c>
       <c r="D19" s="8">
-        <f>((('returns'!$B6*(1+D15))*A19)-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'returns'!$B5</f>
+        <f>((('returns'!$B10*(1+D15))*A19)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
         <v/>
       </c>
       <c r="E19" s="8">
-        <f>((('returns'!$B6*(1+E15))*A19)-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'returns'!$B5</f>
+        <f>((('returns'!$B10*(1+E15))*A19)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
         <v/>
       </c>
       <c r="F19" s="8">
-        <f>((('returns'!$B6*(1+F15))*A19)-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'returns'!$B5</f>
+        <f>((('returns'!$B10*(1+F15))*A19)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
         <v/>
       </c>
     </row>
@@ -3586,23 +3813,23 @@
         <v>11</v>
       </c>
       <c r="B20" s="8">
-        <f>((('returns'!$B6*(1+B15))*A20)-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'returns'!$B5</f>
+        <f>((('returns'!$B10*(1+B15))*A20)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
         <v/>
       </c>
       <c r="C20" s="8">
-        <f>((('returns'!$B6*(1+C15))*A20)-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'returns'!$B5</f>
+        <f>((('returns'!$B10*(1+C15))*A20)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
         <v/>
       </c>
       <c r="D20" s="8">
-        <f>((('returns'!$B6*(1+D15))*A20)-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'returns'!$B5</f>
+        <f>((('returns'!$B10*(1+D15))*A20)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
         <v/>
       </c>
       <c r="E20" s="8">
-        <f>((('returns'!$B6*(1+E15))*A20)-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'returns'!$B5</f>
+        <f>((('returns'!$B10*(1+E15))*A20)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
         <v/>
       </c>
       <c r="F20" s="8">
-        <f>((('returns'!$B6*(1+F15))*A20)-'debt_schedule'!$R8-'debt_schedule'!$S8-'debt_schedule'!$T8+'debt_schedule'!$Q8)/'returns'!$B5</f>
+        <f>((('returns'!$B10*(1+F15))*A20)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
pass 5, second to last debt tranche separation step
</commit_message>
<xml_diff>
--- a/outputs/valuation_model.xlsx
+++ b/outputs/valuation_model.xlsx
@@ -10,13 +10,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cover" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="historicals_input" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="assumptions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sources_uses" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="operating_model" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="debt_schedule" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="returns" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="valuation" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sensitivities" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="checks" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="debt_setup" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sources_uses" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="operating_model" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="debt_schedule" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="returns" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="valuation" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sensitivities" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="checks" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dense_model" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -77,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -85,6 +87,7 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -453,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -517,7 +520,7 @@
         </is>
       </c>
       <c r="B8">
-        <f>'returns'!$B8</f>
+        <f>'returns'!$B9</f>
         <v/>
       </c>
     </row>
@@ -528,7 +531,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>'returns'!$B12</f>
+        <f>'returns'!$B13</f>
         <v/>
       </c>
     </row>
@@ -539,7 +542,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>'returns'!$B20</f>
+        <f>'returns'!$B22</f>
         <v/>
       </c>
     </row>
@@ -550,7 +553,7 @@
         </is>
       </c>
       <c r="B11">
-        <f>'returns'!$B21</f>
+        <f>'returns'!$B23</f>
         <v/>
       </c>
     </row>
@@ -561,7 +564,7 @@
         </is>
       </c>
       <c r="B12">
-        <f>'returns'!$B22</f>
+        <f>'returns'!$B24</f>
         <v/>
       </c>
     </row>
@@ -639,49 +642,63 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>sources_uses</t>
+          <t>debt_setup</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>operating_model</t>
+          <t>sources_uses</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>debt_schedule</t>
+          <t>operating_model</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>returns</t>
+          <t>debt_schedule</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>valuation</t>
+          <t>returns</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>sensitivities</t>
+          <t>valuation</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>sensitivities</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>checks</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>dense_model</t>
         </is>
       </c>
     </row>
@@ -691,6 +708,348 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Sensitivities</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>DCF: WACC vs Terminal Growth</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>WACC \ Growth</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>0.035</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>0.104</v>
+      </c>
+      <c r="B6" s="10">
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A6)^{1,2,3,4,5})+((valuation!I5*(1+B5))/MAX(A6-B5,0.0001))/(1+A6)^5-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'historicals_input'!$B12</f>
+        <v/>
+      </c>
+      <c r="C6" s="10">
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A6)^{1,2,3,4,5})+((valuation!I5*(1+C5))/MAX(A6-C5,0.0001))/(1+A6)^5-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'historicals_input'!$B12</f>
+        <v/>
+      </c>
+      <c r="D6" s="10">
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A6)^{1,2,3,4,5})+((valuation!I5*(1+D5))/MAX(A6-D5,0.0001))/(1+A6)^5-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'historicals_input'!$B12</f>
+        <v/>
+      </c>
+      <c r="E6" s="10">
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A6)^{1,2,3,4,5})+((valuation!I5*(1+E5))/MAX(A6-E5,0.0001))/(1+A6)^5-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'historicals_input'!$B12</f>
+        <v/>
+      </c>
+      <c r="F6" s="10">
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A6)^{1,2,3,4,5})+((valuation!I5*(1+F5))/MAX(A6-F5,0.0001))/(1+A6)^5-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'historicals_input'!$B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>0.109</v>
+      </c>
+      <c r="B7" s="10">
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A7)^{1,2,3,4,5})+((valuation!I5*(1+B5))/MAX(A7-B5,0.0001))/(1+A7)^5-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'historicals_input'!$B12</f>
+        <v/>
+      </c>
+      <c r="C7" s="10">
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A7)^{1,2,3,4,5})+((valuation!I5*(1+C5))/MAX(A7-C5,0.0001))/(1+A7)^5-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'historicals_input'!$B12</f>
+        <v/>
+      </c>
+      <c r="D7" s="10">
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A7)^{1,2,3,4,5})+((valuation!I5*(1+D5))/MAX(A7-D5,0.0001))/(1+A7)^5-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'historicals_input'!$B12</f>
+        <v/>
+      </c>
+      <c r="E7" s="10">
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A7)^{1,2,3,4,5})+((valuation!I5*(1+E5))/MAX(A7-E5,0.0001))/(1+A7)^5-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'historicals_input'!$B12</f>
+        <v/>
+      </c>
+      <c r="F7" s="10">
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A7)^{1,2,3,4,5})+((valuation!I5*(1+F5))/MAX(A7-F5,0.0001))/(1+A7)^5-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'historicals_input'!$B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>0.114</v>
+      </c>
+      <c r="B8" s="10">
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A8)^{1,2,3,4,5})+((valuation!I5*(1+B5))/MAX(A8-B5,0.0001))/(1+A8)^5-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'historicals_input'!$B12</f>
+        <v/>
+      </c>
+      <c r="C8" s="10">
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A8)^{1,2,3,4,5})+((valuation!I5*(1+C5))/MAX(A8-C5,0.0001))/(1+A8)^5-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'historicals_input'!$B12</f>
+        <v/>
+      </c>
+      <c r="D8" s="10">
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A8)^{1,2,3,4,5})+((valuation!I5*(1+D5))/MAX(A8-D5,0.0001))/(1+A8)^5-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'historicals_input'!$B12</f>
+        <v/>
+      </c>
+      <c r="E8" s="10">
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A8)^{1,2,3,4,5})+((valuation!I5*(1+E5))/MAX(A8-E5,0.0001))/(1+A8)^5-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'historicals_input'!$B12</f>
+        <v/>
+      </c>
+      <c r="F8" s="10">
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A8)^{1,2,3,4,5})+((valuation!I5*(1+F5))/MAX(A8-F5,0.0001))/(1+A8)^5-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'historicals_input'!$B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>0.119</v>
+      </c>
+      <c r="B9" s="10">
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A9)^{1,2,3,4,5})+((valuation!I5*(1+B5))/MAX(A9-B5,0.0001))/(1+A9)^5-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'historicals_input'!$B12</f>
+        <v/>
+      </c>
+      <c r="C9" s="10">
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A9)^{1,2,3,4,5})+((valuation!I5*(1+C5))/MAX(A9-C5,0.0001))/(1+A9)^5-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'historicals_input'!$B12</f>
+        <v/>
+      </c>
+      <c r="D9" s="10">
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A9)^{1,2,3,4,5})+((valuation!I5*(1+D5))/MAX(A9-D5,0.0001))/(1+A9)^5-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'historicals_input'!$B12</f>
+        <v/>
+      </c>
+      <c r="E9" s="10">
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A9)^{1,2,3,4,5})+((valuation!I5*(1+E5))/MAX(A9-E5,0.0001))/(1+A9)^5-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'historicals_input'!$B12</f>
+        <v/>
+      </c>
+      <c r="F9" s="10">
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A9)^{1,2,3,4,5})+((valuation!I5*(1+F5))/MAX(A9-F5,0.0001))/(1+A9)^5-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'historicals_input'!$B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>0.124</v>
+      </c>
+      <c r="B10" s="10">
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A10)^{1,2,3,4,5})+((valuation!I5*(1+B5))/MAX(A10-B5,0.0001))/(1+A10)^5-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'historicals_input'!$B12</f>
+        <v/>
+      </c>
+      <c r="C10" s="10">
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A10)^{1,2,3,4,5})+((valuation!I5*(1+C5))/MAX(A10-C5,0.0001))/(1+A10)^5-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'historicals_input'!$B12</f>
+        <v/>
+      </c>
+      <c r="D10" s="10">
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A10)^{1,2,3,4,5})+((valuation!I5*(1+D5))/MAX(A10-D5,0.0001))/(1+A10)^5-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'historicals_input'!$B12</f>
+        <v/>
+      </c>
+      <c r="E10" s="10">
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A10)^{1,2,3,4,5})+((valuation!I5*(1+E5))/MAX(A10-E5,0.0001))/(1+A10)^5-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'historicals_input'!$B12</f>
+        <v/>
+      </c>
+      <c r="F10" s="10">
+        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A10)^{1,2,3,4,5})+((valuation!I5*(1+F5))/MAX(A10-F5,0.0001))/(1+A10)^5-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'historicals_input'!$B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>LBO: Exit Multiple vs Exit EBITDA Adj.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Exit Multiple \ EBITDA Adj.</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>9</v>
+      </c>
+      <c r="B16" s="9">
+        <f>((('returns'!$B11*(1+B15))*A16)-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'returns'!$B9</f>
+        <v/>
+      </c>
+      <c r="C16" s="9">
+        <f>((('returns'!$B11*(1+C15))*A16)-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'returns'!$B9</f>
+        <v/>
+      </c>
+      <c r="D16" s="9">
+        <f>((('returns'!$B11*(1+D15))*A16)-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'returns'!$B9</f>
+        <v/>
+      </c>
+      <c r="E16" s="9">
+        <f>((('returns'!$B11*(1+E15))*A16)-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'returns'!$B9</f>
+        <v/>
+      </c>
+      <c r="F16" s="9">
+        <f>((('returns'!$B11*(1+F15))*A16)-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'returns'!$B9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="B17" s="9">
+        <f>((('returns'!$B11*(1+B15))*A17)-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'returns'!$B9</f>
+        <v/>
+      </c>
+      <c r="C17" s="9">
+        <f>((('returns'!$B11*(1+C15))*A17)-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'returns'!$B9</f>
+        <v/>
+      </c>
+      <c r="D17" s="9">
+        <f>((('returns'!$B11*(1+D15))*A17)-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'returns'!$B9</f>
+        <v/>
+      </c>
+      <c r="E17" s="9">
+        <f>((('returns'!$B11*(1+E15))*A17)-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'returns'!$B9</f>
+        <v/>
+      </c>
+      <c r="F17" s="9">
+        <f>((('returns'!$B11*(1+F15))*A17)-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'returns'!$B9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>10</v>
+      </c>
+      <c r="B18" s="9">
+        <f>((('returns'!$B11*(1+B15))*A18)-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'returns'!$B9</f>
+        <v/>
+      </c>
+      <c r="C18" s="9">
+        <f>((('returns'!$B11*(1+C15))*A18)-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'returns'!$B9</f>
+        <v/>
+      </c>
+      <c r="D18" s="9">
+        <f>((('returns'!$B11*(1+D15))*A18)-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'returns'!$B9</f>
+        <v/>
+      </c>
+      <c r="E18" s="9">
+        <f>((('returns'!$B11*(1+E15))*A18)-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'returns'!$B9</f>
+        <v/>
+      </c>
+      <c r="F18" s="9">
+        <f>((('returns'!$B11*(1+F15))*A18)-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'returns'!$B9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="B19" s="9">
+        <f>((('returns'!$B11*(1+B15))*A19)-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'returns'!$B9</f>
+        <v/>
+      </c>
+      <c r="C19" s="9">
+        <f>((('returns'!$B11*(1+C15))*A19)-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'returns'!$B9</f>
+        <v/>
+      </c>
+      <c r="D19" s="9">
+        <f>((('returns'!$B11*(1+D15))*A19)-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'returns'!$B9</f>
+        <v/>
+      </c>
+      <c r="E19" s="9">
+        <f>((('returns'!$B11*(1+E15))*A19)-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'returns'!$B9</f>
+        <v/>
+      </c>
+      <c r="F19" s="9">
+        <f>((('returns'!$B11*(1+F15))*A19)-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'returns'!$B9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>11</v>
+      </c>
+      <c r="B20" s="9">
+        <f>((('returns'!$B11*(1+B15))*A20)-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'returns'!$B9</f>
+        <v/>
+      </c>
+      <c r="C20" s="9">
+        <f>((('returns'!$B11*(1+C15))*A20)-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'returns'!$B9</f>
+        <v/>
+      </c>
+      <c r="D20" s="9">
+        <f>((('returns'!$B11*(1+D15))*A20)-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'returns'!$B9</f>
+        <v/>
+      </c>
+      <c r="E20" s="9">
+        <f>((('returns'!$B11*(1+E15))*A20)-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'returns'!$B9</f>
+        <v/>
+      </c>
+      <c r="F20" s="9">
+        <f>((('returns'!$B11*(1+F15))*A20)-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8)/'returns'!$B9</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -737,7 +1096,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>ABS('sources_uses'!$B18-'sources_uses'!$B10)</f>
+        <f>ABS('sources_uses'!$B20-'sources_uses'!$B10)</f>
         <v/>
       </c>
       <c r="C4">
@@ -752,7 +1111,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>'sources_uses'!$B17</f>
+        <f>'sources_uses'!$B19</f>
         <v/>
       </c>
       <c r="C5">
@@ -767,7 +1126,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>MIN('debt_schedule'!$T4,'debt_schedule'!$T5,'debt_schedule'!$T6,'debt_schedule'!$T7,'debt_schedule'!$T8)-'historicals_input'!$B19</f>
+        <f>MIN('debt_schedule'!$W4,'debt_schedule'!$W5,'debt_schedule'!$W6,'debt_schedule'!$W7,'debt_schedule'!$W8)-'historicals_input'!$B22</f>
         <v/>
       </c>
       <c r="C6">
@@ -782,7 +1141,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>MIN('debt_schedule'!$U4,'debt_schedule'!$U5,'debt_schedule'!$U6,'debt_schedule'!$U7,'debt_schedule'!$U8)</f>
+        <f>MIN('debt_schedule'!$X$4+'debt_schedule'!$Y$4,'debt_schedule'!$X$5+'debt_schedule'!$Y$5,'debt_schedule'!$X$6+'debt_schedule'!$Y$6,'debt_schedule'!$X$7+'debt_schedule'!$Y$7,'debt_schedule'!$X$8+'debt_schedule'!$Y$8)</f>
         <v/>
       </c>
       <c r="C7">
@@ -797,7 +1156,7 @@
         </is>
       </c>
       <c r="B8">
-        <f>MIN('debt_schedule'!$V4,'debt_schedule'!$V5,'debt_schedule'!$V6,'debt_schedule'!$V7,'debt_schedule'!$V8)</f>
+        <f>MIN('debt_schedule'!$Z4,'debt_schedule'!$Z5,'debt_schedule'!$Z6,'debt_schedule'!$Z7,'debt_schedule'!$Z8)</f>
         <v/>
       </c>
       <c r="C8">
@@ -812,7 +1171,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>'valuation'!$B14-'historicals_input'!$B38</f>
+        <f>'valuation'!$B14-'historicals_input'!$B44</f>
         <v/>
       </c>
       <c r="C9">
@@ -827,7 +1186,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>'returns'!$B20</f>
+        <f>'returns'!$B22</f>
         <v/>
       </c>
       <c r="C10">
@@ -857,7 +1216,7 @@
         </is>
       </c>
       <c r="B12">
-        <f>MAX('debt_schedule'!$S4,'debt_schedule'!$S5,'debt_schedule'!$S6,'debt_schedule'!$S7,'debt_schedule'!$S8)</f>
+        <f>MAX('debt_schedule'!$V4,'debt_schedule'!$V5,'debt_schedule'!$V6,'debt_schedule'!$V7,'debt_schedule'!$V8)</f>
         <v/>
       </c>
       <c r="C12">
@@ -872,7 +1231,7 @@
         </is>
       </c>
       <c r="B13">
-        <f>MAX('debt_schedule'!$W4,'debt_schedule'!$W5,'debt_schedule'!$W6,'debt_schedule'!$W7,'debt_schedule'!$W8)-'historicals_input'!$B28</f>
+        <f>MAX('debt_schedule'!$AA4,'debt_schedule'!$AA5,'debt_schedule'!$AA6,'debt_schedule'!$AA7,'debt_schedule'!$AA8)-'historicals_input'!$B34</f>
         <v/>
       </c>
       <c r="C13">
@@ -944,6 +1303,463 @@
       </c>
       <c r="D19">
         <f>C19-B19</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="2" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Dense Model Snapshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Transaction Summary</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Operating Model</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>2025E</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>2026E</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>2027E</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>2028E</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>2029E</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Purchase Price</t>
+        </is>
+      </c>
+      <c r="B5">
+        <f>'sources_uses'!$B5</f>
+        <v/>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="E5">
+        <f>operating_model!B4</f>
+        <v/>
+      </c>
+      <c r="F5">
+        <f>operating_model!C4</f>
+        <v/>
+      </c>
+      <c r="G5">
+        <f>operating_model!D4</f>
+        <v/>
+      </c>
+      <c r="H5">
+        <f>operating_model!E4</f>
+        <v/>
+      </c>
+      <c r="I5">
+        <f>operating_model!F4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Refinanced Debt</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>'sources_uses'!$B6</f>
+        <v/>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="E6">
+        <f>operating_model!B7</f>
+        <v/>
+      </c>
+      <c r="F6">
+        <f>operating_model!C7</f>
+        <v/>
+      </c>
+      <c r="G6">
+        <f>operating_model!D7</f>
+        <v/>
+      </c>
+      <c r="H6">
+        <f>operating_model!E7</f>
+        <v/>
+      </c>
+      <c r="I6">
+        <f>operating_model!F7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sponsor Equity</t>
+        </is>
+      </c>
+      <c r="B7">
+        <f>'sources_uses'!$B19</f>
+        <v/>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>UFCF</t>
+        </is>
+      </c>
+      <c r="E7">
+        <f>operating_model!B17</f>
+        <v/>
+      </c>
+      <c r="F7">
+        <f>operating_model!C17</f>
+        <v/>
+      </c>
+      <c r="G7">
+        <f>operating_model!D17</f>
+        <v/>
+      </c>
+      <c r="H7">
+        <f>operating_model!E17</f>
+        <v/>
+      </c>
+      <c r="I7">
+        <f>operating_model!F17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Entry EV</t>
+        </is>
+      </c>
+      <c r="B8">
+        <f>'returns'!$B4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Exit EV</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>'returns'!$B13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Exit Equity</t>
+        </is>
+      </c>
+      <c r="B10">
+        <f>'returns'!$B22</f>
+        <v/>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Debt Roll-Forward</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>MOIC</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>'returns'!$B23</f>
+        <v/>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>2025E</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>2026E</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>2027E</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>2028E</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>2029E</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>IRR</t>
+        </is>
+      </c>
+      <c r="B12">
+        <f>'returns'!$B24</f>
+        <v/>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>End TLA</t>
+        </is>
+      </c>
+      <c r="E12">
+        <f>debt_schedule!X4</f>
+        <v/>
+      </c>
+      <c r="F12">
+        <f>debt_schedule!X5</f>
+        <v/>
+      </c>
+      <c r="G12">
+        <f>debt_schedule!X6</f>
+        <v/>
+      </c>
+      <c r="H12">
+        <f>debt_schedule!X7</f>
+        <v/>
+      </c>
+      <c r="I12">
+        <f>debt_schedule!X8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>DCF Share Price</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>'valuation'!$E21</f>
+        <v/>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>End TLB</t>
+        </is>
+      </c>
+      <c r="E13">
+        <f>debt_schedule!Y4</f>
+        <v/>
+      </c>
+      <c r="F13">
+        <f>debt_schedule!Y5</f>
+        <v/>
+      </c>
+      <c r="G13">
+        <f>debt_schedule!Y6</f>
+        <v/>
+      </c>
+      <c r="H13">
+        <f>debt_schedule!Y7</f>
+        <v/>
+      </c>
+      <c r="I13">
+        <f>debt_schedule!Y8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>End Sub Debt</t>
+        </is>
+      </c>
+      <c r="E14">
+        <f>debt_schedule!Z4</f>
+        <v/>
+      </c>
+      <c r="F14">
+        <f>debt_schedule!Z5</f>
+        <v/>
+      </c>
+      <c r="G14">
+        <f>debt_schedule!Z6</f>
+        <v/>
+      </c>
+      <c r="H14">
+        <f>debt_schedule!Z7</f>
+        <v/>
+      </c>
+      <c r="I14">
+        <f>debt_schedule!Z8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>End Revolver</t>
+        </is>
+      </c>
+      <c r="E15">
+        <f>debt_schedule!AA4</f>
+        <v/>
+      </c>
+      <c r="F15">
+        <f>debt_schedule!AA5</f>
+        <v/>
+      </c>
+      <c r="G15">
+        <f>debt_schedule!AA6</f>
+        <v/>
+      </c>
+      <c r="H15">
+        <f>debt_schedule!AA7</f>
+        <v/>
+      </c>
+      <c r="I15">
+        <f>debt_schedule!AA8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>End Cash</t>
+        </is>
+      </c>
+      <c r="E16">
+        <f>debt_schedule!W4</f>
+        <v/>
+      </c>
+      <c r="F16">
+        <f>debt_schedule!W5</f>
+        <v/>
+      </c>
+      <c r="G16">
+        <f>debt_schedule!W6</f>
+        <v/>
+      </c>
+      <c r="H16">
+        <f>debt_schedule!W7</f>
+        <v/>
+      </c>
+      <c r="I16">
+        <f>debt_schedule!W8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Sensitivity Snapshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Avg DCF Matrix</t>
+        </is>
+      </c>
+      <c r="E19">
+        <f>AVERAGE(sensitivities!B6:F10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Avg LBO Matrix</t>
+        </is>
+      </c>
+      <c r="E20">
+        <f>AVERAGE(sensitivities!B16:F20)</f>
         <v/>
       </c>
     </row>
@@ -958,10 +1774,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="23" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
@@ -1145,226 +1961,286 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Existing Debt</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="n">
-        <v>23336000000</v>
+          <t>Debt-Free Acquisition (0/1)</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Existing Cash</t>
+          <t>Existing Debt</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>1000000000</v>
+        <v>23336000000</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Transaction Fee %</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="n">
-        <v>0.02</v>
+          <t>Existing Cash</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>1000000000</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Financing Fee %</t>
+          <t>Transaction Fee %</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Minimum Cash Balance</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="n">
-        <v>50000000</v>
-      </c>
-    </row>
-    <row r="20"/>
+          <t>Financing Fee %</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>OID %</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Financing Assumptions</t>
-        </is>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Management Rollover %</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Senior Debt / EBITDA</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Sub Debt / EBITDA</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
+          <t>Minimum Cash Balance</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>50000000</v>
+      </c>
+    </row>
+    <row r="23"/>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Senior Interest Rate</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="n">
-        <v>0.06</v>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Financing Assumptions</t>
+        </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Sub Interest Rate</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="n">
-        <v>0.08</v>
+          <t>Senior Debt / EBITDA</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Sub PIK Rate</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="n">
-        <v>0</v>
+          <t>Sub Debt / EBITDA</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Revolver Rate</t>
+          <t>Senior Interest Rate</t>
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Revolver Limit</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="n">
-        <v>6255000000</v>
+          <t>Senior Term %</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>0.7</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Senior Amortization %</t>
+          <t>Senior TLA %</t>
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>0.05</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Cash Sweep %</t>
+          <t>Senior TLB %</t>
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31"/>
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Sub Interest Rate</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0.08</v>
+      </c>
+    </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Valuation Assumptions</t>
-        </is>
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Sub PIK Rate</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Tax Rate</t>
+          <t>Revolver Rate</t>
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>0.25</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Risk Free Rate</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="n">
-        <v>0.042</v>
+          <t>Revolver Limit</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="n">
+        <v>6255000000</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Beta</t>
-        </is>
-      </c>
-      <c r="B35" s="7" t="n">
-        <v>1.2</v>
+          <t>Senior Amortization %</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0.05</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Market Risk Premium</t>
+          <t>Cash Sweep %</t>
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>0.06</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Cost of Debt</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="n">
-        <v>0.065</v>
-      </c>
-    </row>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37"/>
     <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Terminal Growth</t>
-        </is>
-      </c>
-      <c r="B38" s="5" t="n">
-        <v>0.025</v>
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Valuation Assumptions</t>
+        </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>Tax Rate</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Risk Free Rate</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0.042</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Beta</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Market Risk Premium</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Cost of Debt</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0.065</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Terminal Growth</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0.025</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>Exit Multiple</t>
         </is>
       </c>
-      <c r="B39" s="6" t="n">
+      <c r="B45" s="6" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1558,17 +2434,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Sources &amp; Uses</t>
+          <t>Debt Tranche Setup</t>
         </is>
       </c>
     </row>
@@ -1576,161 +2455,204 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Uses</t>
+          <t>Debt Tranches</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Line Item</t>
+          <t>Metric</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Amount</t>
+          <t>TLA</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>TLB</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Sub Notes</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Revolver</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Purchase Price</t>
-        </is>
-      </c>
-      <c r="B5" s="4">
-        <f>'historicals_input'!$B13*'historicals_input'!$B14</f>
+          <t>Target Multiple</t>
+        </is>
+      </c>
+      <c r="B5">
+        <f>'historicals_input'!$B25*'historicals_input'!$B29</f>
+        <v/>
+      </c>
+      <c r="C5">
+        <f>'historicals_input'!$B25*'historicals_input'!$B30</f>
+        <v/>
+      </c>
+      <c r="D5">
+        <f>'historicals_input'!$B26</f>
+        <v/>
+      </c>
+      <c r="E5">
+        <f>IFERROR('historicals_input'!$B34/'historicals_input'!$B13,0)</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Refinance Existing Debt</t>
-        </is>
-      </c>
-      <c r="B6" s="4">
-        <f>'historicals_input'!$B15</f>
+          <t>Gross Debt</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>'historicals_input'!$B13*B5</f>
+        <v/>
+      </c>
+      <c r="C6">
+        <f>'historicals_input'!$B13*C5</f>
+        <v/>
+      </c>
+      <c r="D6">
+        <f>'historicals_input'!$B13*D5</f>
+        <v/>
+      </c>
+      <c r="E6">
+        <f>'historicals_input'!$B34</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Transaction Fees</t>
-        </is>
-      </c>
-      <c r="B7" s="4">
-        <f>B5*'historicals_input'!$B17</f>
-        <v/>
+          <t>OID %</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="C7">
+        <f>'historicals_input'!$B20</f>
+        <v/>
+      </c>
+      <c r="D7">
+        <f>'historicals_input'!$B20</f>
+        <v/>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Financing Fees</t>
-        </is>
-      </c>
-      <c r="B8" s="4">
-        <f>(B11+B12)*'historicals_input'!$B18</f>
+          <t>Net Funding</t>
+        </is>
+      </c>
+      <c r="B8">
+        <f>B6*(1-B7)</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>C6*(1-C7)</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>D6*(1-D7)</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>0</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Minimum Cash</t>
-        </is>
-      </c>
-      <c r="B9" s="4">
-        <f>'historicals_input'!$B19</f>
+          <t>Cash Interest Rate</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>'historicals_input'!$B27</f>
+        <v/>
+      </c>
+      <c r="C9">
+        <f>'historicals_input'!$B27</f>
+        <v/>
+      </c>
+      <c r="D9">
+        <f>'historicals_input'!$B31</f>
+        <v/>
+      </c>
+      <c r="E9">
+        <f>'historicals_input'!$B33</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Total Uses</t>
-        </is>
-      </c>
-      <c r="B10" s="4">
-        <f>SUM(B5:B9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11"/>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Sources</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Line Item</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Senior Debt</t>
-        </is>
-      </c>
-      <c r="B14" s="4">
-        <f>'historicals_input'!$B13*'historicals_input'!$B22</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Sub Debt</t>
-        </is>
-      </c>
-      <c r="B15" s="4">
-        <f>'historicals_input'!$B13*'historicals_input'!$B23</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Existing Cash</t>
-        </is>
-      </c>
-      <c r="B16" s="4">
-        <f>'historicals_input'!$B16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Sponsor Equity</t>
-        </is>
-      </c>
-      <c r="B17" s="4">
-        <f>B10-SUM(B14:B16)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Total Sources</t>
-        </is>
-      </c>
-      <c r="B18" s="4">
-        <f>SUM(B14:B17)</f>
-        <v/>
+          <t>PIK Rate</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="D10">
+        <f>'historicals_input'!$B32</f>
+        <v/>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Amortization %</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>'historicals_input'!$B35</f>
+        <v/>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1739,6 +2661,277 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="2" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Sources &amp; Uses</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Uses</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Capital Structure Bridge</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Line Item</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Purchase Price</t>
+        </is>
+      </c>
+      <c r="B5" s="4">
+        <f>'historicals_input'!$B13*'historicals_input'!$B14</f>
+        <v/>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Gross TLA</t>
+        </is>
+      </c>
+      <c r="E5" s="4">
+        <f>'debt_setup'!$B6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Refinance Existing Debt</t>
+        </is>
+      </c>
+      <c r="B6" s="4">
+        <f>(1-'historicals_input'!$B15)*'historicals_input'!$B16</f>
+        <v/>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Gross TLB</t>
+        </is>
+      </c>
+      <c r="E6" s="4">
+        <f>'debt_setup'!$C6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Transaction Fees</t>
+        </is>
+      </c>
+      <c r="B7" s="4">
+        <f>B5*'historicals_input'!$B18</f>
+        <v/>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Gross Sub</t>
+        </is>
+      </c>
+      <c r="E7" s="4">
+        <f>'debt_setup'!$D6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Financing Fees</t>
+        </is>
+      </c>
+      <c r="B8" s="4">
+        <f>('debt_setup'!$B6+'debt_setup'!$C6+'debt_setup'!$D6)*'historicals_input'!$B19</f>
+        <v/>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>OID Discount</t>
+        </is>
+      </c>
+      <c r="E8" s="4">
+        <f>SUM(E5:E7)-SUM(B14:B16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Minimum Cash</t>
+        </is>
+      </c>
+      <c r="B9" s="4">
+        <f>'historicals_input'!$B22</f>
+        <v/>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Total Net New Debt</t>
+        </is>
+      </c>
+      <c r="E9" s="4">
+        <f>SUM(B14:B16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Total Uses</t>
+        </is>
+      </c>
+      <c r="B10" s="4">
+        <f>SUM(B5:B9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Line Item</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TLA Net Debt</t>
+        </is>
+      </c>
+      <c r="B14" s="4">
+        <f>'debt_setup'!$B8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>TLB Net Debt</t>
+        </is>
+      </c>
+      <c r="B15" s="4">
+        <f>'debt_setup'!$C8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Sub Debt</t>
+        </is>
+      </c>
+      <c r="B16" s="4">
+        <f>'debt_setup'!$D8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Existing Cash</t>
+        </is>
+      </c>
+      <c r="B17" s="4">
+        <f>'historicals_input'!$B17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Management Rollover</t>
+        </is>
+      </c>
+      <c r="B18" s="4">
+        <f>B5*'historicals_input'!$B21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Sponsor Equity</t>
+        </is>
+      </c>
+      <c r="B19" s="4">
+        <f>B10-SUM(B14:B18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Total Sources</t>
+        </is>
+      </c>
+      <c r="B20" s="4">
+        <f>SUM(B14:B19)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2003,23 +3196,23 @@
         </is>
       </c>
       <c r="B11" s="4">
-        <f>B10*'historicals_input'!$B33</f>
+        <f>B10*'historicals_input'!$B39</f>
         <v/>
       </c>
       <c r="C11" s="4">
-        <f>C10*'historicals_input'!$B33</f>
+        <f>C10*'historicals_input'!$B39</f>
         <v/>
       </c>
       <c r="D11" s="4">
-        <f>D10*'historicals_input'!$B33</f>
+        <f>D10*'historicals_input'!$B39</f>
         <v/>
       </c>
       <c r="E11" s="4">
-        <f>E10*'historicals_input'!$B33</f>
+        <f>E10*'historicals_input'!$B39</f>
         <v/>
       </c>
       <c r="F11" s="4">
-        <f>F10*'historicals_input'!$B33</f>
+        <f>F10*'historicals_input'!$B39</f>
         <v/>
       </c>
     </row>
@@ -2182,634 +3375,6 @@
       </c>
       <c r="F17" s="4">
         <f>F10-F11+F9-F13-F16</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:W8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="26" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
-    <col width="23" customWidth="1" min="11" max="11"/>
-    <col width="26" customWidth="1" min="12" max="12"/>
-    <col width="26" customWidth="1" min="13" max="13"/>
-    <col width="21" customWidth="1" min="14" max="14"/>
-    <col width="26" customWidth="1" min="15" max="15"/>
-    <col width="23" customWidth="1" min="16" max="16"/>
-    <col width="26" customWidth="1" min="17" max="17"/>
-    <col width="26" customWidth="1" min="18" max="18"/>
-    <col width="26" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="18" customWidth="1" min="21" max="21"/>
-    <col width="18" customWidth="1" min="22" max="22"/>
-    <col width="18" customWidth="1" min="23" max="23"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Debt Schedule</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Year</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Beg Cash</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Beg Senior</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Beg Sub</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Beg Revolver</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>UFCF</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Senior Interest</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>Sub Cash Interest</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>Sub PIK</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>Revolver Interest</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>Cash Pre Debt Service</t>
-        </is>
-      </c>
-      <c r="L3" s="3" t="inlineStr">
-        <is>
-          <t>Mandatory Senior</t>
-        </is>
-      </c>
-      <c r="M3" s="3" t="inlineStr">
-        <is>
-          <t>Revolver Repay</t>
-        </is>
-      </c>
-      <c r="N3" s="3" t="inlineStr">
-        <is>
-          <t>Cash Post Mandatory</t>
-        </is>
-      </c>
-      <c r="O3" s="3" t="inlineStr">
-        <is>
-          <t>Cash Sweep Capacity</t>
-        </is>
-      </c>
-      <c r="P3" s="3" t="inlineStr">
-        <is>
-          <t>Senior Sweep</t>
-        </is>
-      </c>
-      <c r="Q3" s="3" t="inlineStr">
-        <is>
-          <t>Sub Sweep</t>
-        </is>
-      </c>
-      <c r="R3" s="3" t="inlineStr">
-        <is>
-          <t>Revolver Draw</t>
-        </is>
-      </c>
-      <c r="S3" s="3" t="inlineStr">
-        <is>
-          <t>Liquidity Shortfall</t>
-        </is>
-      </c>
-      <c r="T3" s="3" t="inlineStr">
-        <is>
-          <t>End Cash</t>
-        </is>
-      </c>
-      <c r="U3" s="3" t="inlineStr">
-        <is>
-          <t>End Senior</t>
-        </is>
-      </c>
-      <c r="V3" s="3" t="inlineStr">
-        <is>
-          <t>End Sub</t>
-        </is>
-      </c>
-      <c r="W3" s="3" t="inlineStr">
-        <is>
-          <t>End Revolver</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B4" s="4">
-        <f>'sources_uses'!$B9</f>
-        <v/>
-      </c>
-      <c r="C4" s="4">
-        <f>'sources_uses'!$B14</f>
-        <v/>
-      </c>
-      <c r="D4" s="4">
-        <f>'sources_uses'!$B15</f>
-        <v/>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="4">
-        <f>'operating_model'!$B17</f>
-        <v/>
-      </c>
-      <c r="G4" s="4">
-        <f>C4*'historicals_input'!$B24</f>
-        <v/>
-      </c>
-      <c r="H4" s="4">
-        <f>D4*'historicals_input'!$B25</f>
-        <v/>
-      </c>
-      <c r="I4" s="4">
-        <f>D4*'historicals_input'!$B26</f>
-        <v/>
-      </c>
-      <c r="J4" s="4">
-        <f>E4*'historicals_input'!$B27</f>
-        <v/>
-      </c>
-      <c r="K4" s="4">
-        <f>B4+F4-G4-H4-J4</f>
-        <v/>
-      </c>
-      <c r="L4" s="4">
-        <f>MIN(C4*'historicals_input'!$B29,C4)</f>
-        <v/>
-      </c>
-      <c r="M4" s="4">
-        <f>MIN(MAX(K4-L4-'historicals_input'!$B19,0),E4)</f>
-        <v/>
-      </c>
-      <c r="N4" s="4">
-        <f>K4-L4-M4</f>
-        <v/>
-      </c>
-      <c r="O4" s="4">
-        <f>MAX(N4-'historicals_input'!$B19,0)*'historicals_input'!$B30</f>
-        <v/>
-      </c>
-      <c r="P4" s="4">
-        <f>MIN(O4,MAX(C4-L4,0))</f>
-        <v/>
-      </c>
-      <c r="Q4" s="4">
-        <f>MIN(MAX(O4-P4,0),D4+I4)</f>
-        <v/>
-      </c>
-      <c r="R4" s="4">
-        <f>MIN(MAX('historicals_input'!$B19-(N4-P4-Q4),0),MAX('historicals_input'!$B28-E4+M4,0))</f>
-        <v/>
-      </c>
-      <c r="S4" s="4">
-        <f>MAX('historicals_input'!$B19-(N4-P4-Q4-R4),0)</f>
-        <v/>
-      </c>
-      <c r="T4" s="4">
-        <f>N4-P4-Q4+R4</f>
-        <v/>
-      </c>
-      <c r="U4" s="4">
-        <f>MAX(C4-L4-P4,0)</f>
-        <v/>
-      </c>
-      <c r="V4" s="4">
-        <f>MAX(D4+I4-Q4,0)</f>
-        <v/>
-      </c>
-      <c r="W4" s="4">
-        <f>MAX(E4-M4+R4,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B5" s="4">
-        <f>T4</f>
-        <v/>
-      </c>
-      <c r="C5" s="4">
-        <f>U4</f>
-        <v/>
-      </c>
-      <c r="D5" s="4">
-        <f>V4</f>
-        <v/>
-      </c>
-      <c r="E5" s="4">
-        <f>W4</f>
-        <v/>
-      </c>
-      <c r="F5" s="4">
-        <f>'operating_model'!$C17</f>
-        <v/>
-      </c>
-      <c r="G5" s="4">
-        <f>C5*'historicals_input'!$B24</f>
-        <v/>
-      </c>
-      <c r="H5" s="4">
-        <f>D5*'historicals_input'!$B25</f>
-        <v/>
-      </c>
-      <c r="I5" s="4">
-        <f>D5*'historicals_input'!$B26</f>
-        <v/>
-      </c>
-      <c r="J5" s="4">
-        <f>E5*'historicals_input'!$B27</f>
-        <v/>
-      </c>
-      <c r="K5" s="4">
-        <f>B5+F5-G5-H5-J5</f>
-        <v/>
-      </c>
-      <c r="L5" s="4">
-        <f>MIN(C5*'historicals_input'!$B29,C5)</f>
-        <v/>
-      </c>
-      <c r="M5" s="4">
-        <f>MIN(MAX(K5-L5-'historicals_input'!$B19,0),E5)</f>
-        <v/>
-      </c>
-      <c r="N5" s="4">
-        <f>K5-L5-M5</f>
-        <v/>
-      </c>
-      <c r="O5" s="4">
-        <f>MAX(N5-'historicals_input'!$B19,0)*'historicals_input'!$B30</f>
-        <v/>
-      </c>
-      <c r="P5" s="4">
-        <f>MIN(O5,MAX(C5-L5,0))</f>
-        <v/>
-      </c>
-      <c r="Q5" s="4">
-        <f>MIN(MAX(O5-P5,0),D5+I5)</f>
-        <v/>
-      </c>
-      <c r="R5" s="4">
-        <f>MIN(MAX('historicals_input'!$B19-(N5-P5-Q5),0),MAX('historicals_input'!$B28-E5+M5,0))</f>
-        <v/>
-      </c>
-      <c r="S5" s="4">
-        <f>MAX('historicals_input'!$B19-(N5-P5-Q5-R5),0)</f>
-        <v/>
-      </c>
-      <c r="T5" s="4">
-        <f>N5-P5-Q5+R5</f>
-        <v/>
-      </c>
-      <c r="U5" s="4">
-        <f>MAX(C5-L5-P5,0)</f>
-        <v/>
-      </c>
-      <c r="V5" s="4">
-        <f>MAX(D5+I5-Q5,0)</f>
-        <v/>
-      </c>
-      <c r="W5" s="4">
-        <f>MAX(E5-M5+R5,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>2027</v>
-      </c>
-      <c r="B6" s="4">
-        <f>T5</f>
-        <v/>
-      </c>
-      <c r="C6" s="4">
-        <f>U5</f>
-        <v/>
-      </c>
-      <c r="D6" s="4">
-        <f>V5</f>
-        <v/>
-      </c>
-      <c r="E6" s="4">
-        <f>W5</f>
-        <v/>
-      </c>
-      <c r="F6" s="4">
-        <f>'operating_model'!$D17</f>
-        <v/>
-      </c>
-      <c r="G6" s="4">
-        <f>C6*'historicals_input'!$B24</f>
-        <v/>
-      </c>
-      <c r="H6" s="4">
-        <f>D6*'historicals_input'!$B25</f>
-        <v/>
-      </c>
-      <c r="I6" s="4">
-        <f>D6*'historicals_input'!$B26</f>
-        <v/>
-      </c>
-      <c r="J6" s="4">
-        <f>E6*'historicals_input'!$B27</f>
-        <v/>
-      </c>
-      <c r="K6" s="4">
-        <f>B6+F6-G6-H6-J6</f>
-        <v/>
-      </c>
-      <c r="L6" s="4">
-        <f>MIN(C6*'historicals_input'!$B29,C6)</f>
-        <v/>
-      </c>
-      <c r="M6" s="4">
-        <f>MIN(MAX(K6-L6-'historicals_input'!$B19,0),E6)</f>
-        <v/>
-      </c>
-      <c r="N6" s="4">
-        <f>K6-L6-M6</f>
-        <v/>
-      </c>
-      <c r="O6" s="4">
-        <f>MAX(N6-'historicals_input'!$B19,0)*'historicals_input'!$B30</f>
-        <v/>
-      </c>
-      <c r="P6" s="4">
-        <f>MIN(O6,MAX(C6-L6,0))</f>
-        <v/>
-      </c>
-      <c r="Q6" s="4">
-        <f>MIN(MAX(O6-P6,0),D6+I6)</f>
-        <v/>
-      </c>
-      <c r="R6" s="4">
-        <f>MIN(MAX('historicals_input'!$B19-(N6-P6-Q6),0),MAX('historicals_input'!$B28-E6+M6,0))</f>
-        <v/>
-      </c>
-      <c r="S6" s="4">
-        <f>MAX('historicals_input'!$B19-(N6-P6-Q6-R6),0)</f>
-        <v/>
-      </c>
-      <c r="T6" s="4">
-        <f>N6-P6-Q6+R6</f>
-        <v/>
-      </c>
-      <c r="U6" s="4">
-        <f>MAX(C6-L6-P6,0)</f>
-        <v/>
-      </c>
-      <c r="V6" s="4">
-        <f>MAX(D6+I6-Q6,0)</f>
-        <v/>
-      </c>
-      <c r="W6" s="4">
-        <f>MAX(E6-M6+R6,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>2028</v>
-      </c>
-      <c r="B7" s="4">
-        <f>T6</f>
-        <v/>
-      </c>
-      <c r="C7" s="4">
-        <f>U6</f>
-        <v/>
-      </c>
-      <c r="D7" s="4">
-        <f>V6</f>
-        <v/>
-      </c>
-      <c r="E7" s="4">
-        <f>W6</f>
-        <v/>
-      </c>
-      <c r="F7" s="4">
-        <f>'operating_model'!$E17</f>
-        <v/>
-      </c>
-      <c r="G7" s="4">
-        <f>C7*'historicals_input'!$B24</f>
-        <v/>
-      </c>
-      <c r="H7" s="4">
-        <f>D7*'historicals_input'!$B25</f>
-        <v/>
-      </c>
-      <c r="I7" s="4">
-        <f>D7*'historicals_input'!$B26</f>
-        <v/>
-      </c>
-      <c r="J7" s="4">
-        <f>E7*'historicals_input'!$B27</f>
-        <v/>
-      </c>
-      <c r="K7" s="4">
-        <f>B7+F7-G7-H7-J7</f>
-        <v/>
-      </c>
-      <c r="L7" s="4">
-        <f>MIN(C7*'historicals_input'!$B29,C7)</f>
-        <v/>
-      </c>
-      <c r="M7" s="4">
-        <f>MIN(MAX(K7-L7-'historicals_input'!$B19,0),E7)</f>
-        <v/>
-      </c>
-      <c r="N7" s="4">
-        <f>K7-L7-M7</f>
-        <v/>
-      </c>
-      <c r="O7" s="4">
-        <f>MAX(N7-'historicals_input'!$B19,0)*'historicals_input'!$B30</f>
-        <v/>
-      </c>
-      <c r="P7" s="4">
-        <f>MIN(O7,MAX(C7-L7,0))</f>
-        <v/>
-      </c>
-      <c r="Q7" s="4">
-        <f>MIN(MAX(O7-P7,0),D7+I7)</f>
-        <v/>
-      </c>
-      <c r="R7" s="4">
-        <f>MIN(MAX('historicals_input'!$B19-(N7-P7-Q7),0),MAX('historicals_input'!$B28-E7+M7,0))</f>
-        <v/>
-      </c>
-      <c r="S7" s="4">
-        <f>MAX('historicals_input'!$B19-(N7-P7-Q7-R7),0)</f>
-        <v/>
-      </c>
-      <c r="T7" s="4">
-        <f>N7-P7-Q7+R7</f>
-        <v/>
-      </c>
-      <c r="U7" s="4">
-        <f>MAX(C7-L7-P7,0)</f>
-        <v/>
-      </c>
-      <c r="V7" s="4">
-        <f>MAX(D7+I7-Q7,0)</f>
-        <v/>
-      </c>
-      <c r="W7" s="4">
-        <f>MAX(E7-M7+R7,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>2029</v>
-      </c>
-      <c r="B8" s="4">
-        <f>T7</f>
-        <v/>
-      </c>
-      <c r="C8" s="4">
-        <f>U7</f>
-        <v/>
-      </c>
-      <c r="D8" s="4">
-        <f>V7</f>
-        <v/>
-      </c>
-      <c r="E8" s="4">
-        <f>W7</f>
-        <v/>
-      </c>
-      <c r="F8" s="4">
-        <f>'operating_model'!$F17</f>
-        <v/>
-      </c>
-      <c r="G8" s="4">
-        <f>C8*'historicals_input'!$B24</f>
-        <v/>
-      </c>
-      <c r="H8" s="4">
-        <f>D8*'historicals_input'!$B25</f>
-        <v/>
-      </c>
-      <c r="I8" s="4">
-        <f>D8*'historicals_input'!$B26</f>
-        <v/>
-      </c>
-      <c r="J8" s="4">
-        <f>E8*'historicals_input'!$B27</f>
-        <v/>
-      </c>
-      <c r="K8" s="4">
-        <f>B8+F8-G8-H8-J8</f>
-        <v/>
-      </c>
-      <c r="L8" s="4">
-        <f>MIN(C8*'historicals_input'!$B29,C8)</f>
-        <v/>
-      </c>
-      <c r="M8" s="4">
-        <f>MIN(MAX(K8-L8-'historicals_input'!$B19,0),E8)</f>
-        <v/>
-      </c>
-      <c r="N8" s="4">
-        <f>K8-L8-M8</f>
-        <v/>
-      </c>
-      <c r="O8" s="4">
-        <f>MAX(N8-'historicals_input'!$B19,0)*'historicals_input'!$B30</f>
-        <v/>
-      </c>
-      <c r="P8" s="4">
-        <f>MIN(O8,MAX(C8-L8,0))</f>
-        <v/>
-      </c>
-      <c r="Q8" s="4">
-        <f>MIN(MAX(O8-P8,0),D8+I8)</f>
-        <v/>
-      </c>
-      <c r="R8" s="4">
-        <f>MIN(MAX('historicals_input'!$B19-(N8-P8-Q8),0),MAX('historicals_input'!$B28-E8+M8,0))</f>
-        <v/>
-      </c>
-      <c r="S8" s="4">
-        <f>MAX('historicals_input'!$B19-(N8-P8-Q8-R8),0)</f>
-        <v/>
-      </c>
-      <c r="T8" s="4">
-        <f>N8-P8-Q8+R8</f>
-        <v/>
-      </c>
-      <c r="U8" s="4">
-        <f>MAX(C8-L8-P8,0)</f>
-        <v/>
-      </c>
-      <c r="V8" s="4">
-        <f>MAX(D8+I8-Q8,0)</f>
-        <v/>
-      </c>
-      <c r="W8" s="4">
-        <f>MAX(E8-M8+R8,0)</f>
         <v/>
       </c>
     </row>
@@ -2824,7 +3389,739 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:AA8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="23" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="14" max="14"/>
+    <col width="26" customWidth="1" min="15" max="15"/>
+    <col width="21" customWidth="1" min="16" max="16"/>
+    <col width="26" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="26" customWidth="1" min="19" max="19"/>
+    <col width="26" customWidth="1" min="20" max="20"/>
+    <col width="26" customWidth="1" min="21" max="21"/>
+    <col width="26" customWidth="1" min="22" max="22"/>
+    <col width="17" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="15" customWidth="1" min="25" max="25"/>
+    <col width="18" customWidth="1" min="26" max="26"/>
+    <col width="18" customWidth="1" min="27" max="27"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Debt Schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Beg Cash</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Beg TLA</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Beg TLB</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Beg Sub</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Beg Revolver</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>UFCF</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>TLA Interest</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>TLB Interest</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Sub Cash Interest</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>Sub PIK</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>Revolver Interest</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>Cash Pre Debt Service</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>TLA Mandatory</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>Revolver Repay</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>Cash Post Mandatory</t>
+        </is>
+      </c>
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>Cash Sweep Capacity</t>
+        </is>
+      </c>
+      <c r="R3" s="3" t="inlineStr">
+        <is>
+          <t>TLB Sweep</t>
+        </is>
+      </c>
+      <c r="S3" s="3" t="inlineStr">
+        <is>
+          <t>TLA Sweep</t>
+        </is>
+      </c>
+      <c r="T3" s="3" t="inlineStr">
+        <is>
+          <t>Sub Sweep</t>
+        </is>
+      </c>
+      <c r="U3" s="3" t="inlineStr">
+        <is>
+          <t>Revolver Draw</t>
+        </is>
+      </c>
+      <c r="V3" s="3" t="inlineStr">
+        <is>
+          <t>Liquidity Shortfall</t>
+        </is>
+      </c>
+      <c r="W3" s="3" t="inlineStr">
+        <is>
+          <t>End Cash</t>
+        </is>
+      </c>
+      <c r="X3" s="3" t="inlineStr">
+        <is>
+          <t>End TLA</t>
+        </is>
+      </c>
+      <c r="Y3" s="3" t="inlineStr">
+        <is>
+          <t>End TLB</t>
+        </is>
+      </c>
+      <c r="Z3" s="3" t="inlineStr">
+        <is>
+          <t>End Sub</t>
+        </is>
+      </c>
+      <c r="AA3" s="3" t="inlineStr">
+        <is>
+          <t>End Revolver</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B4" s="4">
+        <f>'sources_uses'!$B9</f>
+        <v/>
+      </c>
+      <c r="C4" s="4">
+        <f>'sources_uses'!$B$14</f>
+        <v/>
+      </c>
+      <c r="D4" s="4">
+        <f>'sources_uses'!$B$15</f>
+        <v/>
+      </c>
+      <c r="E4" s="4">
+        <f>'sources_uses'!$B16</f>
+        <v/>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="4">
+        <f>'operating_model'!$B17</f>
+        <v/>
+      </c>
+      <c r="H4" s="4">
+        <f>C4*'debt_setup'!$B9</f>
+        <v/>
+      </c>
+      <c r="I4" s="4">
+        <f>D4*'debt_setup'!$C9</f>
+        <v/>
+      </c>
+      <c r="J4" s="4">
+        <f>E4*'historicals_input'!$B31</f>
+        <v/>
+      </c>
+      <c r="K4" s="4">
+        <f>E4*'historicals_input'!$B32</f>
+        <v/>
+      </c>
+      <c r="L4" s="4">
+        <f>F4*'historicals_input'!$B33</f>
+        <v/>
+      </c>
+      <c r="M4" s="4">
+        <f>B4+G4-H4-I4-J4-L4</f>
+        <v/>
+      </c>
+      <c r="N4" s="4">
+        <f>MIN(C4*'debt_setup'!$B11,C4)</f>
+        <v/>
+      </c>
+      <c r="O4" s="4">
+        <f>MIN(MAX(M4-N4-'historicals_input'!$B22,0),F4)</f>
+        <v/>
+      </c>
+      <c r="P4" s="4">
+        <f>M4-N4-O4</f>
+        <v/>
+      </c>
+      <c r="Q4" s="4">
+        <f>MAX(P4-'historicals_input'!$B22,0)*'historicals_input'!$B36</f>
+        <v/>
+      </c>
+      <c r="R4" s="4">
+        <f>MIN(Q4,D4)</f>
+        <v/>
+      </c>
+      <c r="S4" s="4">
+        <f>MIN(MAX(Q4-R4,0),MAX(C4-N4,0))</f>
+        <v/>
+      </c>
+      <c r="T4" s="4">
+        <f>MIN(MAX(Q4-R4-S4,0),E4+K4)</f>
+        <v/>
+      </c>
+      <c r="U4" s="4">
+        <f>MIN(MAX('historicals_input'!$B22-(P4-R4-S4-T4),0),MAX('historicals_input'!$B34-F4+O4,0))</f>
+        <v/>
+      </c>
+      <c r="V4" s="4">
+        <f>MAX('historicals_input'!$B22-(P4-R4-S4-T4-U4),0)</f>
+        <v/>
+      </c>
+      <c r="W4" s="4">
+        <f>P4-R4-S4-T4+U4</f>
+        <v/>
+      </c>
+      <c r="X4" s="4">
+        <f>MAX(C4-N4-S4,0)</f>
+        <v/>
+      </c>
+      <c r="Y4" s="4">
+        <f>MAX(D4-R4,0)</f>
+        <v/>
+      </c>
+      <c r="Z4" s="4">
+        <f>MAX(E4+K4-T4,0)</f>
+        <v/>
+      </c>
+      <c r="AA4" s="4">
+        <f>MAX(F4-O4+U4,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B5" s="4">
+        <f>U4</f>
+        <v/>
+      </c>
+      <c r="C5" s="4">
+        <f>V4</f>
+        <v/>
+      </c>
+      <c r="D5" s="4">
+        <f>W4</f>
+        <v/>
+      </c>
+      <c r="E5" s="4">
+        <f>X4</f>
+        <v/>
+      </c>
+      <c r="F5" s="4">
+        <f>Y4</f>
+        <v/>
+      </c>
+      <c r="G5" s="4">
+        <f>'operating_model'!$C17</f>
+        <v/>
+      </c>
+      <c r="H5" s="4">
+        <f>C5*'debt_setup'!$B9</f>
+        <v/>
+      </c>
+      <c r="I5" s="4">
+        <f>D5*'debt_setup'!$C9</f>
+        <v/>
+      </c>
+      <c r="J5" s="4">
+        <f>E5*'historicals_input'!$B31</f>
+        <v/>
+      </c>
+      <c r="K5" s="4">
+        <f>E5*'historicals_input'!$B32</f>
+        <v/>
+      </c>
+      <c r="L5" s="4">
+        <f>F5*'historicals_input'!$B33</f>
+        <v/>
+      </c>
+      <c r="M5" s="4">
+        <f>B5+G5-H5-I5-J5-L5</f>
+        <v/>
+      </c>
+      <c r="N5" s="4">
+        <f>MIN(C5*'debt_setup'!$B11,C5)</f>
+        <v/>
+      </c>
+      <c r="O5" s="4">
+        <f>MIN(MAX(M5-N5-'historicals_input'!$B22,0),F5)</f>
+        <v/>
+      </c>
+      <c r="P5" s="4">
+        <f>M5-N5-O5</f>
+        <v/>
+      </c>
+      <c r="Q5" s="4">
+        <f>MAX(P5-'historicals_input'!$B22,0)*'historicals_input'!$B36</f>
+        <v/>
+      </c>
+      <c r="R5" s="4">
+        <f>MIN(Q5,D5)</f>
+        <v/>
+      </c>
+      <c r="S5" s="4">
+        <f>MIN(MAX(Q5-R5,0),MAX(C5-N5,0))</f>
+        <v/>
+      </c>
+      <c r="T5" s="4">
+        <f>MIN(MAX(Q5-R5-S5,0),E5+K5)</f>
+        <v/>
+      </c>
+      <c r="U5" s="4">
+        <f>MIN(MAX('historicals_input'!$B22-(P5-R5-S5-T5),0),MAX('historicals_input'!$B34-F5+O5,0))</f>
+        <v/>
+      </c>
+      <c r="V5" s="4">
+        <f>MAX('historicals_input'!$B22-(P5-R5-S5-T5-U5),0)</f>
+        <v/>
+      </c>
+      <c r="W5" s="4">
+        <f>P5-R5-S5-T5+U5</f>
+        <v/>
+      </c>
+      <c r="X5" s="4">
+        <f>MAX(C5-N5-S5,0)</f>
+        <v/>
+      </c>
+      <c r="Y5" s="4">
+        <f>MAX(D5-R5,0)</f>
+        <v/>
+      </c>
+      <c r="Z5" s="4">
+        <f>MAX(E5+K5-T5,0)</f>
+        <v/>
+      </c>
+      <c r="AA5" s="4">
+        <f>MAX(F5-O5+U5,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B6" s="4">
+        <f>U5</f>
+        <v/>
+      </c>
+      <c r="C6" s="4">
+        <f>V5</f>
+        <v/>
+      </c>
+      <c r="D6" s="4">
+        <f>W5</f>
+        <v/>
+      </c>
+      <c r="E6" s="4">
+        <f>X5</f>
+        <v/>
+      </c>
+      <c r="F6" s="4">
+        <f>Y5</f>
+        <v/>
+      </c>
+      <c r="G6" s="4">
+        <f>'operating_model'!$D17</f>
+        <v/>
+      </c>
+      <c r="H6" s="4">
+        <f>C6*'debt_setup'!$B9</f>
+        <v/>
+      </c>
+      <c r="I6" s="4">
+        <f>D6*'debt_setup'!$C9</f>
+        <v/>
+      </c>
+      <c r="J6" s="4">
+        <f>E6*'historicals_input'!$B31</f>
+        <v/>
+      </c>
+      <c r="K6" s="4">
+        <f>E6*'historicals_input'!$B32</f>
+        <v/>
+      </c>
+      <c r="L6" s="4">
+        <f>F6*'historicals_input'!$B33</f>
+        <v/>
+      </c>
+      <c r="M6" s="4">
+        <f>B6+G6-H6-I6-J6-L6</f>
+        <v/>
+      </c>
+      <c r="N6" s="4">
+        <f>MIN(C6*'debt_setup'!$B11,C6)</f>
+        <v/>
+      </c>
+      <c r="O6" s="4">
+        <f>MIN(MAX(M6-N6-'historicals_input'!$B22,0),F6)</f>
+        <v/>
+      </c>
+      <c r="P6" s="4">
+        <f>M6-N6-O6</f>
+        <v/>
+      </c>
+      <c r="Q6" s="4">
+        <f>MAX(P6-'historicals_input'!$B22,0)*'historicals_input'!$B36</f>
+        <v/>
+      </c>
+      <c r="R6" s="4">
+        <f>MIN(Q6,D6)</f>
+        <v/>
+      </c>
+      <c r="S6" s="4">
+        <f>MIN(MAX(Q6-R6,0),MAX(C6-N6,0))</f>
+        <v/>
+      </c>
+      <c r="T6" s="4">
+        <f>MIN(MAX(Q6-R6-S6,0),E6+K6)</f>
+        <v/>
+      </c>
+      <c r="U6" s="4">
+        <f>MIN(MAX('historicals_input'!$B22-(P6-R6-S6-T6),0),MAX('historicals_input'!$B34-F6+O6,0))</f>
+        <v/>
+      </c>
+      <c r="V6" s="4">
+        <f>MAX('historicals_input'!$B22-(P6-R6-S6-T6-U6),0)</f>
+        <v/>
+      </c>
+      <c r="W6" s="4">
+        <f>P6-R6-S6-T6+U6</f>
+        <v/>
+      </c>
+      <c r="X6" s="4">
+        <f>MAX(C6-N6-S6,0)</f>
+        <v/>
+      </c>
+      <c r="Y6" s="4">
+        <f>MAX(D6-R6,0)</f>
+        <v/>
+      </c>
+      <c r="Z6" s="4">
+        <f>MAX(E6+K6-T6,0)</f>
+        <v/>
+      </c>
+      <c r="AA6" s="4">
+        <f>MAX(F6-O6+U6,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2028</v>
+      </c>
+      <c r="B7" s="4">
+        <f>U6</f>
+        <v/>
+      </c>
+      <c r="C7" s="4">
+        <f>V6</f>
+        <v/>
+      </c>
+      <c r="D7" s="4">
+        <f>W6</f>
+        <v/>
+      </c>
+      <c r="E7" s="4">
+        <f>X6</f>
+        <v/>
+      </c>
+      <c r="F7" s="4">
+        <f>Y6</f>
+        <v/>
+      </c>
+      <c r="G7" s="4">
+        <f>'operating_model'!$E17</f>
+        <v/>
+      </c>
+      <c r="H7" s="4">
+        <f>C7*'debt_setup'!$B9</f>
+        <v/>
+      </c>
+      <c r="I7" s="4">
+        <f>D7*'debt_setup'!$C9</f>
+        <v/>
+      </c>
+      <c r="J7" s="4">
+        <f>E7*'historicals_input'!$B31</f>
+        <v/>
+      </c>
+      <c r="K7" s="4">
+        <f>E7*'historicals_input'!$B32</f>
+        <v/>
+      </c>
+      <c r="L7" s="4">
+        <f>F7*'historicals_input'!$B33</f>
+        <v/>
+      </c>
+      <c r="M7" s="4">
+        <f>B7+G7-H7-I7-J7-L7</f>
+        <v/>
+      </c>
+      <c r="N7" s="4">
+        <f>MIN(C7*'debt_setup'!$B11,C7)</f>
+        <v/>
+      </c>
+      <c r="O7" s="4">
+        <f>MIN(MAX(M7-N7-'historicals_input'!$B22,0),F7)</f>
+        <v/>
+      </c>
+      <c r="P7" s="4">
+        <f>M7-N7-O7</f>
+        <v/>
+      </c>
+      <c r="Q7" s="4">
+        <f>MAX(P7-'historicals_input'!$B22,0)*'historicals_input'!$B36</f>
+        <v/>
+      </c>
+      <c r="R7" s="4">
+        <f>MIN(Q7,D7)</f>
+        <v/>
+      </c>
+      <c r="S7" s="4">
+        <f>MIN(MAX(Q7-R7,0),MAX(C7-N7,0))</f>
+        <v/>
+      </c>
+      <c r="T7" s="4">
+        <f>MIN(MAX(Q7-R7-S7,0),E7+K7)</f>
+        <v/>
+      </c>
+      <c r="U7" s="4">
+        <f>MIN(MAX('historicals_input'!$B22-(P7-R7-S7-T7),0),MAX('historicals_input'!$B34-F7+O7,0))</f>
+        <v/>
+      </c>
+      <c r="V7" s="4">
+        <f>MAX('historicals_input'!$B22-(P7-R7-S7-T7-U7),0)</f>
+        <v/>
+      </c>
+      <c r="W7" s="4">
+        <f>P7-R7-S7-T7+U7</f>
+        <v/>
+      </c>
+      <c r="X7" s="4">
+        <f>MAX(C7-N7-S7,0)</f>
+        <v/>
+      </c>
+      <c r="Y7" s="4">
+        <f>MAX(D7-R7,0)</f>
+        <v/>
+      </c>
+      <c r="Z7" s="4">
+        <f>MAX(E7+K7-T7,0)</f>
+        <v/>
+      </c>
+      <c r="AA7" s="4">
+        <f>MAX(F7-O7+U7,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2029</v>
+      </c>
+      <c r="B8" s="4">
+        <f>U7</f>
+        <v/>
+      </c>
+      <c r="C8" s="4">
+        <f>V7</f>
+        <v/>
+      </c>
+      <c r="D8" s="4">
+        <f>W7</f>
+        <v/>
+      </c>
+      <c r="E8" s="4">
+        <f>X7</f>
+        <v/>
+      </c>
+      <c r="F8" s="4">
+        <f>Y7</f>
+        <v/>
+      </c>
+      <c r="G8" s="4">
+        <f>'operating_model'!$F17</f>
+        <v/>
+      </c>
+      <c r="H8" s="4">
+        <f>C8*'debt_setup'!$B9</f>
+        <v/>
+      </c>
+      <c r="I8" s="4">
+        <f>D8*'debt_setup'!$C9</f>
+        <v/>
+      </c>
+      <c r="J8" s="4">
+        <f>E8*'historicals_input'!$B31</f>
+        <v/>
+      </c>
+      <c r="K8" s="4">
+        <f>E8*'historicals_input'!$B32</f>
+        <v/>
+      </c>
+      <c r="L8" s="4">
+        <f>F8*'historicals_input'!$B33</f>
+        <v/>
+      </c>
+      <c r="M8" s="4">
+        <f>B8+G8-H8-I8-J8-L8</f>
+        <v/>
+      </c>
+      <c r="N8" s="4">
+        <f>MIN(C8*'debt_setup'!$B11,C8)</f>
+        <v/>
+      </c>
+      <c r="O8" s="4">
+        <f>MIN(MAX(M8-N8-'historicals_input'!$B22,0),F8)</f>
+        <v/>
+      </c>
+      <c r="P8" s="4">
+        <f>M8-N8-O8</f>
+        <v/>
+      </c>
+      <c r="Q8" s="4">
+        <f>MAX(P8-'historicals_input'!$B22,0)*'historicals_input'!$B36</f>
+        <v/>
+      </c>
+      <c r="R8" s="4">
+        <f>MIN(Q8,D8)</f>
+        <v/>
+      </c>
+      <c r="S8" s="4">
+        <f>MIN(MAX(Q8-R8,0),MAX(C8-N8,0))</f>
+        <v/>
+      </c>
+      <c r="T8" s="4">
+        <f>MIN(MAX(Q8-R8-S8,0),E8+K8)</f>
+        <v/>
+      </c>
+      <c r="U8" s="4">
+        <f>MIN(MAX('historicals_input'!$B22-(P8-R8-S8-T8),0),MAX('historicals_input'!$B34-F8+O8,0))</f>
+        <v/>
+      </c>
+      <c r="V8" s="4">
+        <f>MAX('historicals_input'!$B22-(P8-R8-S8-T8-U8),0)</f>
+        <v/>
+      </c>
+      <c r="W8" s="4">
+        <f>P8-R8-S8-T8+U8</f>
+        <v/>
+      </c>
+      <c r="X8" s="4">
+        <f>MAX(C8-N8-S8,0)</f>
+        <v/>
+      </c>
+      <c r="Y8" s="4">
+        <f>MAX(D8-R8,0)</f>
+        <v/>
+      </c>
+      <c r="Z8" s="4">
+        <f>MAX(E8+K8-T8,0)</f>
+        <v/>
+      </c>
+      <c r="AA8" s="4">
+        <f>MAX(F8-O8+U8,0)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -2865,220 +4162,242 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Entry Senior Debt</t>
+          <t>Entry TLA Debt</t>
         </is>
       </c>
       <c r="B5" s="4">
-        <f>'sources_uses'!$B14</f>
+        <f>'sources_uses'!$B$14</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Entry Sub Debt</t>
+          <t>Entry TLB Debt</t>
         </is>
       </c>
       <c r="B6" s="4">
-        <f>'sources_uses'!$B15</f>
+        <f>'sources_uses'!$B$15</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Entry Net Debt</t>
+          <t>Entry Sub Debt</t>
         </is>
       </c>
       <c r="B7" s="4">
-        <f>B5+B6</f>
+        <f>'sources_uses'!$B16</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Sponsor Equity</t>
+          <t>Entry Net Debt</t>
         </is>
       </c>
       <c r="B8" s="4">
-        <f>'sources_uses'!$B17</f>
+        <f>SUM(B5:B7)</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Entry Debt / EBITDA</t>
-        </is>
-      </c>
-      <c r="B9" s="8">
-        <f>IFERROR(B7/'historicals_input'!$B13,0)</f>
+          <t>Sponsor Equity</t>
+        </is>
+      </c>
+      <c r="B9" s="4">
+        <f>'sources_uses'!$B19</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Exit EBITDA</t>
-        </is>
-      </c>
-      <c r="B10" s="4">
-        <f>'operating_model'!$F7</f>
+          <t>Entry Debt / EBITDA</t>
+        </is>
+      </c>
+      <c r="B10" s="9">
+        <f>IFERROR(B8/'historicals_input'!$B13,0)</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Exit Multiple</t>
-        </is>
-      </c>
-      <c r="B11" s="6">
-        <f>'historicals_input'!$B39</f>
+          <t>Exit EBITDA</t>
+        </is>
+      </c>
+      <c r="B11" s="4">
+        <f>'operating_model'!$F7</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Exit EV</t>
-        </is>
-      </c>
-      <c r="B12" s="4">
-        <f>B10*B11</f>
+          <t>Exit Multiple</t>
+        </is>
+      </c>
+      <c r="B12" s="6">
+        <f>'historicals_input'!$B45</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Exit Senior Debt</t>
+          <t>Exit EV</t>
         </is>
       </c>
       <c r="B13" s="4">
-        <f>'debt_schedule'!$U8</f>
+        <f>B11*B12</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Exit Sub Debt</t>
+          <t>Exit TLA Debt</t>
         </is>
       </c>
       <c r="B14" s="4">
-        <f>'debt_schedule'!$V8</f>
+        <f>'debt_schedule'!$X8</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Exit Revolver</t>
+          <t>Exit TLB Debt</t>
         </is>
       </c>
       <c r="B15" s="4">
-        <f>'debt_schedule'!$W8</f>
+        <f>'debt_schedule'!$Y8</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Exit Cash</t>
+          <t>Exit Sub Debt</t>
         </is>
       </c>
       <c r="B16" s="4">
-        <f>'debt_schedule'!$T8</f>
+        <f>'debt_schedule'!$Z8</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Exit Net Debt</t>
+          <t>Exit Revolver</t>
         </is>
       </c>
       <c r="B17" s="4">
-        <f>B13+B14+B15-B16</f>
+        <f>'debt_schedule'!$AA8</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Exit Debt / EBITDA</t>
-        </is>
-      </c>
-      <c r="B18" s="8">
-        <f>IFERROR(B17/B10,0)</f>
+          <t>Exit Cash</t>
+        </is>
+      </c>
+      <c r="B18" s="4">
+        <f>'debt_schedule'!$W8</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Debt Paydown</t>
+          <t>Exit Net Debt</t>
         </is>
       </c>
       <c r="B19" s="4">
-        <f>B7-B17</f>
+        <f>SUM(B14:B17)-B18</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Exit Equity Value</t>
-        </is>
-      </c>
-      <c r="B20" s="4">
-        <f>B12-B13-B14-B15+B16</f>
+          <t>Exit Debt / EBITDA</t>
+        </is>
+      </c>
+      <c r="B20" s="9">
+        <f>IFERROR(B19/B11,0)</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MOIC</t>
-        </is>
-      </c>
-      <c r="B21" s="8">
-        <f>IFERROR(B20/B8,0)</f>
+          <t>Debt Paydown</t>
+        </is>
+      </c>
+      <c r="B21" s="4">
+        <f>B8-B19</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>IRR</t>
-        </is>
-      </c>
-      <c r="B22" s="5">
-        <f>IFERROR(B21^(1/5)-1,0)</f>
+          <t>Exit Equity Value</t>
+        </is>
+      </c>
+      <c r="B22" s="4">
+        <f>B13-SUM(B14:B17)+B18</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Revenue CAGR</t>
-        </is>
-      </c>
-      <c r="B23" s="5">
-        <f>IFERROR((operating_model!F4/historicals_input!B7)^(1/5)-1,0)</f>
+          <t>MOIC</t>
+        </is>
+      </c>
+      <c r="B23" s="9">
+        <f>IFERROR(B22/B9,0)</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>IRR</t>
+        </is>
+      </c>
+      <c r="B24" s="5">
+        <f>IFERROR(B23^(1/5)-1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Revenue CAGR</t>
+        </is>
+      </c>
+      <c r="B25" s="5">
+        <f>IFERROR((operating_model!F4/historicals_input!B7)^(1/5)-1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>EBITDA CAGR</t>
         </is>
       </c>
-      <c r="B24" s="5">
-        <f>IFERROR((B10/historicals_input!C7)^(1/5)-1,0)</f>
+      <c r="B26" s="5">
+        <f>IFERROR((B11/historicals_input!C7)^(1/5)-1,0)</f>
         <v/>
       </c>
     </row>
@@ -3087,7 +4406,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3182,7 +4501,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>'historicals_input'!$B34</f>
+        <f>'historicals_input'!$B40</f>
         <v/>
       </c>
       <c r="D5" t="inlineStr">
@@ -3217,8 +4536,8 @@
           <t>Beta</t>
         </is>
       </c>
-      <c r="B6" s="7">
-        <f>'historicals_input'!$B35</f>
+      <c r="B6" s="8">
+        <f>'historicals_input'!$B41</f>
         <v/>
       </c>
       <c r="D6" t="inlineStr">
@@ -3254,7 +4573,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>'historicals_input'!$B36</f>
+        <f>'historicals_input'!$B42</f>
         <v/>
       </c>
       <c r="D7" t="inlineStr">
@@ -3301,7 +4620,7 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>'historicals_input'!$B37</f>
+        <f>'historicals_input'!$B43</f>
         <v/>
       </c>
       <c r="D9" t="inlineStr">
@@ -3310,7 +4629,7 @@
         </is>
       </c>
       <c r="E9">
-        <f>'historicals_input'!$B38</f>
+        <f>'historicals_input'!$B44</f>
         <v/>
       </c>
     </row>
@@ -3321,7 +4640,7 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>'historicals_input'!$B33</f>
+        <f>'historicals_input'!$B39</f>
         <v/>
       </c>
       <c r="D10" t="inlineStr">
@@ -3330,7 +4649,7 @@
         </is>
       </c>
       <c r="E10">
-        <f>'historicals_input'!$B39</f>
+        <f>'historicals_input'!$B45</f>
         <v/>
       </c>
     </row>
@@ -3361,7 +4680,7 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>'returns'!$B8/('returns'!$B8+'sources_uses'!$B14+'sources_uses'!$B15)</f>
+        <f>'returns'!$B9/('returns'!$B9+'sources_uses'!$B$14+'sources_uses'!$B$15+'sources_uses'!$B16)</f>
         <v/>
       </c>
       <c r="D12" t="inlineStr">
@@ -3454,7 +4773,7 @@
         </is>
       </c>
       <c r="E18" s="4">
-        <f>E16-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8</f>
+        <f>E16-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8</f>
         <v/>
       </c>
     </row>
@@ -3465,7 +4784,7 @@
         </is>
       </c>
       <c r="E19" s="4">
-        <f>E17-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8</f>
+        <f>E17-'debt_schedule'!$X$8+'debt_schedule'!$Y$8-'debt_schedule'!$Z8-'debt_schedule'!$AA8+'debt_schedule'!$W8</f>
         <v/>
       </c>
     </row>
@@ -3475,7 +4794,7 @@
           <t>Share Price (PGR)</t>
         </is>
       </c>
-      <c r="E20" s="9">
+      <c r="E20" s="10">
         <f>E18/'historicals_input'!$B12</f>
         <v/>
       </c>
@@ -3486,350 +4805,8 @@
           <t>Share Price (Multiple)</t>
         </is>
       </c>
-      <c r="E21" s="9">
+      <c r="E21" s="10">
         <f>E19/'historicals_input'!$B12</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Sensitivities</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>DCF: WACC vs Terminal Growth</t>
-        </is>
-      </c>
-    </row>
-    <row r="4"/>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>WACC \ Growth</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>0.025</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="F5" s="3" t="n">
-        <v>0.035</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>0.104</v>
-      </c>
-      <c r="B6" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A6)^{1,2,3,4,5})+((valuation!I5*(1+B5))/MAX(A6-B5,0.0001))/(1+A6)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
-        <v/>
-      </c>
-      <c r="C6" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A6)^{1,2,3,4,5})+((valuation!I5*(1+C5))/MAX(A6-C5,0.0001))/(1+A6)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
-        <v/>
-      </c>
-      <c r="D6" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A6)^{1,2,3,4,5})+((valuation!I5*(1+D5))/MAX(A6-D5,0.0001))/(1+A6)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
-        <v/>
-      </c>
-      <c r="E6" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A6)^{1,2,3,4,5})+((valuation!I5*(1+E5))/MAX(A6-E5,0.0001))/(1+A6)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
-        <v/>
-      </c>
-      <c r="F6" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A6)^{1,2,3,4,5})+((valuation!I5*(1+F5))/MAX(A6-F5,0.0001))/(1+A6)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>0.109</v>
-      </c>
-      <c r="B7" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A7)^{1,2,3,4,5})+((valuation!I5*(1+B5))/MAX(A7-B5,0.0001))/(1+A7)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
-        <v/>
-      </c>
-      <c r="C7" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A7)^{1,2,3,4,5})+((valuation!I5*(1+C5))/MAX(A7-C5,0.0001))/(1+A7)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
-        <v/>
-      </c>
-      <c r="D7" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A7)^{1,2,3,4,5})+((valuation!I5*(1+D5))/MAX(A7-D5,0.0001))/(1+A7)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
-        <v/>
-      </c>
-      <c r="E7" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A7)^{1,2,3,4,5})+((valuation!I5*(1+E5))/MAX(A7-E5,0.0001))/(1+A7)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
-        <v/>
-      </c>
-      <c r="F7" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A7)^{1,2,3,4,5})+((valuation!I5*(1+F5))/MAX(A7-F5,0.0001))/(1+A7)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>0.114</v>
-      </c>
-      <c r="B8" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A8)^{1,2,3,4,5})+((valuation!I5*(1+B5))/MAX(A8-B5,0.0001))/(1+A8)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
-        <v/>
-      </c>
-      <c r="C8" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A8)^{1,2,3,4,5})+((valuation!I5*(1+C5))/MAX(A8-C5,0.0001))/(1+A8)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
-        <v/>
-      </c>
-      <c r="D8" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A8)^{1,2,3,4,5})+((valuation!I5*(1+D5))/MAX(A8-D5,0.0001))/(1+A8)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
-        <v/>
-      </c>
-      <c r="E8" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A8)^{1,2,3,4,5})+((valuation!I5*(1+E5))/MAX(A8-E5,0.0001))/(1+A8)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
-        <v/>
-      </c>
-      <c r="F8" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A8)^{1,2,3,4,5})+((valuation!I5*(1+F5))/MAX(A8-F5,0.0001))/(1+A8)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>0.119</v>
-      </c>
-      <c r="B9" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A9)^{1,2,3,4,5})+((valuation!I5*(1+B5))/MAX(A9-B5,0.0001))/(1+A9)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
-        <v/>
-      </c>
-      <c r="C9" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A9)^{1,2,3,4,5})+((valuation!I5*(1+C5))/MAX(A9-C5,0.0001))/(1+A9)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
-        <v/>
-      </c>
-      <c r="D9" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A9)^{1,2,3,4,5})+((valuation!I5*(1+D5))/MAX(A9-D5,0.0001))/(1+A9)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
-        <v/>
-      </c>
-      <c r="E9" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A9)^{1,2,3,4,5})+((valuation!I5*(1+E5))/MAX(A9-E5,0.0001))/(1+A9)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
-        <v/>
-      </c>
-      <c r="F9" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A9)^{1,2,3,4,5})+((valuation!I5*(1+F5))/MAX(A9-F5,0.0001))/(1+A9)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>0.124</v>
-      </c>
-      <c r="B10" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A10)^{1,2,3,4,5})+((valuation!I5*(1+B5))/MAX(A10-B5,0.0001))/(1+A10)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
-        <v/>
-      </c>
-      <c r="C10" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A10)^{1,2,3,4,5})+((valuation!I5*(1+C5))/MAX(A10-C5,0.0001))/(1+A10)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
-        <v/>
-      </c>
-      <c r="D10" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A10)^{1,2,3,4,5})+((valuation!I5*(1+D5))/MAX(A10-D5,0.0001))/(1+A10)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
-        <v/>
-      </c>
-      <c r="E10" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A10)^{1,2,3,4,5})+((valuation!I5*(1+E5))/MAX(A10-E5,0.0001))/(1+A10)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
-        <v/>
-      </c>
-      <c r="F10" s="9">
-        <f>(SUMPRODUCT(valuation!E5:I5,1/(1+A10)^{1,2,3,4,5})+((valuation!I5*(1+F5))/MAX(A10-F5,0.0001))/(1+A10)^5-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'historicals_input'!$B12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>LBO: Exit Multiple vs Exit EBITDA Adj.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14"/>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Exit Multiple \ EBITDA Adj.</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="n">
-        <v>-0.1</v>
-      </c>
-      <c r="C15" s="3" t="n">
-        <v>-0.05</v>
-      </c>
-      <c r="D15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="3" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="F15" s="3" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>9</v>
-      </c>
-      <c r="B16" s="8">
-        <f>((('returns'!$B10*(1+B15))*A16)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
-        <v/>
-      </c>
-      <c r="C16" s="8">
-        <f>((('returns'!$B10*(1+C15))*A16)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
-        <v/>
-      </c>
-      <c r="D16" s="8">
-        <f>((('returns'!$B10*(1+D15))*A16)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
-        <v/>
-      </c>
-      <c r="E16" s="8">
-        <f>((('returns'!$B10*(1+E15))*A16)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
-        <v/>
-      </c>
-      <c r="F16" s="8">
-        <f>((('returns'!$B10*(1+F15))*A16)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="B17" s="8">
-        <f>((('returns'!$B10*(1+B15))*A17)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
-        <v/>
-      </c>
-      <c r="C17" s="8">
-        <f>((('returns'!$B10*(1+C15))*A17)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
-        <v/>
-      </c>
-      <c r="D17" s="8">
-        <f>((('returns'!$B10*(1+D15))*A17)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
-        <v/>
-      </c>
-      <c r="E17" s="8">
-        <f>((('returns'!$B10*(1+E15))*A17)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
-        <v/>
-      </c>
-      <c r="F17" s="8">
-        <f>((('returns'!$B10*(1+F15))*A17)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>10</v>
-      </c>
-      <c r="B18" s="8">
-        <f>((('returns'!$B10*(1+B15))*A18)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
-        <v/>
-      </c>
-      <c r="C18" s="8">
-        <f>((('returns'!$B10*(1+C15))*A18)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
-        <v/>
-      </c>
-      <c r="D18" s="8">
-        <f>((('returns'!$B10*(1+D15))*A18)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
-        <v/>
-      </c>
-      <c r="E18" s="8">
-        <f>((('returns'!$B10*(1+E15))*A18)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
-        <v/>
-      </c>
-      <c r="F18" s="8">
-        <f>((('returns'!$B10*(1+F15))*A18)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="B19" s="8">
-        <f>((('returns'!$B10*(1+B15))*A19)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
-        <v/>
-      </c>
-      <c r="C19" s="8">
-        <f>((('returns'!$B10*(1+C15))*A19)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
-        <v/>
-      </c>
-      <c r="D19" s="8">
-        <f>((('returns'!$B10*(1+D15))*A19)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
-        <v/>
-      </c>
-      <c r="E19" s="8">
-        <f>((('returns'!$B10*(1+E15))*A19)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
-        <v/>
-      </c>
-      <c r="F19" s="8">
-        <f>((('returns'!$B10*(1+F15))*A19)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>11</v>
-      </c>
-      <c r="B20" s="8">
-        <f>((('returns'!$B10*(1+B15))*A20)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
-        <v/>
-      </c>
-      <c r="C20" s="8">
-        <f>((('returns'!$B10*(1+C15))*A20)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
-        <v/>
-      </c>
-      <c r="D20" s="8">
-        <f>((('returns'!$B10*(1+D15))*A20)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
-        <v/>
-      </c>
-      <c r="E20" s="8">
-        <f>((('returns'!$B10*(1+E15))*A20)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
-        <v/>
-      </c>
-      <c r="F20" s="8">
-        <f>((('returns'!$B10*(1+F15))*A20)-'debt_schedule'!$U8-'debt_schedule'!$V8-'debt_schedule'!$W8+'debt_schedule'!$T8)/'returns'!$B8</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
pass 6, model wired. now going to add extraction pipeline
</commit_message>
<xml_diff>
--- a/outputs/valuation_model.xlsx
+++ b/outputs/valuation_model.xlsx
@@ -3410,12 +3410,12 @@
     <col width="21" customWidth="1" min="16" max="16"/>
     <col width="26" customWidth="1" min="17" max="17"/>
     <col width="13" customWidth="1" min="18" max="18"/>
-    <col width="26" customWidth="1" min="19" max="19"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
     <col width="26" customWidth="1" min="20" max="20"/>
     <col width="26" customWidth="1" min="21" max="21"/>
     <col width="26" customWidth="1" min="22" max="22"/>
     <col width="17" customWidth="1" min="23" max="23"/>
-    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="15" customWidth="1" min="24" max="24"/>
     <col width="15" customWidth="1" min="25" max="25"/>
     <col width="18" customWidth="1" min="26" max="26"/>
     <col width="18" customWidth="1" min="27" max="27"/>
@@ -3638,7 +3638,7 @@
         <v/>
       </c>
       <c r="S4" s="4">
-        <f>MIN(MAX(Q4-R4,0),MAX(C4-N4,0))</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="T4" s="4">
@@ -3658,7 +3658,7 @@
         <v/>
       </c>
       <c r="X4" s="4">
-        <f>MAX(C4-N4-S4,0)</f>
+        <f>MAX(C4-N4,0)</f>
         <v/>
       </c>
       <c r="Y4" s="4">
@@ -3747,7 +3747,7 @@
         <v/>
       </c>
       <c r="S5" s="4">
-        <f>MIN(MAX(Q5-R5,0),MAX(C5-N5,0))</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="T5" s="4">
@@ -3767,7 +3767,7 @@
         <v/>
       </c>
       <c r="X5" s="4">
-        <f>MAX(C5-N5-S5,0)</f>
+        <f>MAX(C5-N5,0)</f>
         <v/>
       </c>
       <c r="Y5" s="4">
@@ -3856,7 +3856,7 @@
         <v/>
       </c>
       <c r="S6" s="4">
-        <f>MIN(MAX(Q6-R6,0),MAX(C6-N6,0))</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="T6" s="4">
@@ -3876,7 +3876,7 @@
         <v/>
       </c>
       <c r="X6" s="4">
-        <f>MAX(C6-N6-S6,0)</f>
+        <f>MAX(C6-N6,0)</f>
         <v/>
       </c>
       <c r="Y6" s="4">
@@ -3965,7 +3965,7 @@
         <v/>
       </c>
       <c r="S7" s="4">
-        <f>MIN(MAX(Q7-R7,0),MAX(C7-N7,0))</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="T7" s="4">
@@ -3985,7 +3985,7 @@
         <v/>
       </c>
       <c r="X7" s="4">
-        <f>MAX(C7-N7-S7,0)</f>
+        <f>MAX(C7-N7,0)</f>
         <v/>
       </c>
       <c r="Y7" s="4">
@@ -4074,7 +4074,7 @@
         <v/>
       </c>
       <c r="S8" s="4">
-        <f>MIN(MAX(Q8-R8,0),MAX(C8-N8,0))</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="T8" s="4">
@@ -4094,7 +4094,7 @@
         <v/>
       </c>
       <c r="X8" s="4">
-        <f>MAX(C8-N8-S8,0)</f>
+        <f>MAX(C8-N8,0)</f>
         <v/>
       </c>
       <c r="Y8" s="4">

</xml_diff>